<commit_message>
docs: sync notes, slides, Gantt, figures and literature review for the Oct 20 meeting
- Project notes: four-stage chain, where things stand section by section,
  task-specific dataset table, October papers, distillation answer
- Slides moved into docs/notes/Slides; Oct 20 deck added
- Gantt workbook: research-plan add-ons slotted as IDs 17, 18, 24, 38,
  41, 42, 43
- Figures: paper figure scripts and the 21 Overleaf PDFs plus PNGs
  (project_logic, blf_pipeline, research_plan, task_coverage redrawn)
- Literature review: new Section 3.4 on fair comparison, alignment as a
  task, and multi-omics benchmarks; Works Cited extended
- sources.md: papers raised in October 2026
- Removed the stray all_figures copy and the meeting video from docs/notes

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016iUz3FrBfCmdjUW7KcJVVN
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -245,6 +245,15 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -519,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z55"/>
+  <dimension ref="A1:Z58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -588,7 +597,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 3, 2026. Fall weeks start Monday; January–March 2027 is an adjustable monthly horizon.</t>
+          <t>As of October 10, 2026. Fall weeks start Monday; January to March 2027 is an adjustable monthly horizon. Rows 41 to 43 and the edits to 17, 18 and 24 fold in the research plan's add-ons.</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1649,7 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Run matched BioLangFusion-style comparisons</t>
+          <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (add-on 1)</t>
         </is>
       </c>
       <c r="C25" s="24" t="inlineStr">
@@ -1655,7 +1664,7 @@
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>Oct 18</t>
+          <t>Oct 25</t>
         </is>
       </c>
       <c r="F25" s="13" t="str"/>
@@ -1668,7 +1677,11 @@
           <t>██</t>
         </is>
       </c>
-      <c r="L25" s="13" t="str"/>
+      <c r="L25" s="24" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="M25" s="13" t="str"/>
       <c r="N25" s="13" t="str"/>
       <c r="O25" s="13" t="str"/>
@@ -1690,7 +1703,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Repeat diagnostics and null/control comparisons</t>
+          <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (add-on 5)</t>
         </is>
       </c>
       <c r="C26" s="24" t="inlineStr">
@@ -2002,12 +2015,12 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Candidate additional DNA, RNA and protein encoder comparisons</t>
-        </is>
-      </c>
-      <c r="C32" s="29" t="inlineStr">
-        <is>
-          <t>Conditional</t>
+          <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (add-on 2)</t>
+        </is>
+      </c>
+      <c r="C32" s="38" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
@@ -2029,7 +2042,7 @@
       <c r="L32" s="13" t="str"/>
       <c r="M32" s="13" t="str"/>
       <c r="N32" s="13" t="str"/>
-      <c r="O32" s="31" t="inlineStr">
+      <c r="O32" s="39" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2328,267 +2341,182 @@
       <c r="Y37" s="13" t="str"/>
       <c r="Z37" s="13" t="str"/>
     </row>
-    <row r="38" ht="29" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>Research writing and coordination</t>
-        </is>
-      </c>
+    <row r="38" ht="41" customHeight="1">
+      <c r="A38" s="13" t="n">
+        <v>41</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>LucaOne frozen baseline on stability and GTEx, matched comparison (add-on 3)</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>Oct 19</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>Nov 1</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="n"/>
+      <c r="G38" s="13" t="n"/>
+      <c r="H38" s="13" t="n"/>
+      <c r="I38" s="13" t="n"/>
+      <c r="J38" s="13" t="n"/>
+      <c r="K38" s="13" t="n"/>
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N38" s="13" t="n"/>
+      <c r="O38" s="13" t="n"/>
+      <c r="P38" s="40" t="n"/>
+      <c r="Q38" s="40" t="n"/>
+      <c r="R38" s="13" t="n"/>
+      <c r="S38" s="13" t="n"/>
+      <c r="T38" s="13" t="n"/>
+      <c r="U38" s="13" t="n"/>
+      <c r="V38" s="13" t="n"/>
+      <c r="W38" s="11" t="n"/>
+      <c r="X38" s="13" t="n"/>
+      <c r="Y38" s="13" t="n"/>
+      <c r="Z38" s="13" t="n"/>
     </row>
     <row r="39" ht="41" customHeight="1">
       <c r="A39" s="13" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Research coordination and decision review</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
+          <t>mRNABench half-life and translation efficiency after the sequence and label gates (add-on 4)</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>Conditional</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>Sep 14</t>
+          <t>Jan 4</t>
         </is>
       </c>
       <c r="E39" s="15" t="inlineStr">
         <is>
-          <t>Mar 31</t>
-        </is>
-      </c>
-      <c r="F39" s="13" t="str"/>
-      <c r="G39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="H39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="J39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="K39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="R39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="S39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="T39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="U39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="V39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+          <t>Feb 28</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="n"/>
+      <c r="G39" s="13" t="n"/>
+      <c r="H39" s="13" t="n"/>
+      <c r="I39" s="13" t="n"/>
+      <c r="J39" s="13" t="n"/>
+      <c r="K39" s="13" t="n"/>
+      <c r="L39" s="13" t="n"/>
+      <c r="M39" s="13" t="n"/>
+      <c r="N39" s="13" t="n"/>
+      <c r="O39" s="13" t="n"/>
+      <c r="P39" s="40" t="n"/>
+      <c r="Q39" s="40" t="n"/>
+      <c r="R39" s="13" t="n"/>
+      <c r="S39" s="13" t="n"/>
+      <c r="T39" s="13" t="n"/>
+      <c r="U39" s="13" t="n"/>
+      <c r="V39" s="13" t="n"/>
       <c r="W39" s="11" t="n"/>
-      <c r="X39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z39" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="X39" s="28" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y39" s="28" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z39" s="13" t="n"/>
     </row>
     <row r="40" ht="41" customHeight="1">
       <c r="A40" s="13" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Maintain and revise the living Overleaf manuscript</t>
-        </is>
-      </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
+          <t>Multi-teacher distillation pilot, RNA first (add-on 7)</t>
+        </is>
+      </c>
+      <c r="C40" s="28" t="inlineStr">
+        <is>
+          <t>Conditional</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Jan 4</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>Mar 31</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="str"/>
-      <c r="G40" s="13" t="str"/>
-      <c r="H40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="R40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="S40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="T40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="U40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="V40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+          <t>Feb 28</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n"/>
+      <c r="G40" s="13" t="n"/>
+      <c r="H40" s="13" t="n"/>
+      <c r="I40" s="13" t="n"/>
+      <c r="J40" s="13" t="n"/>
+      <c r="K40" s="13" t="n"/>
+      <c r="L40" s="13" t="n"/>
+      <c r="M40" s="13" t="n"/>
+      <c r="N40" s="13" t="n"/>
+      <c r="O40" s="13" t="n"/>
+      <c r="P40" s="40" t="n"/>
+      <c r="Q40" s="40" t="n"/>
+      <c r="R40" s="13" t="n"/>
+      <c r="S40" s="13" t="n"/>
+      <c r="T40" s="13" t="n"/>
+      <c r="U40" s="13" t="n"/>
+      <c r="V40" s="13" t="n"/>
       <c r="W40" s="11" t="n"/>
-      <c r="X40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z40" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="X40" s="28" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y40" s="28" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z40" s="13" t="n"/>
     </row>
     <row r="41" ht="29" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>CAP6942 course deliverables</t>
+          <t>Research writing and coordination</t>
         </is>
       </c>
     </row>
     <row r="42" ht="41" customHeight="1">
       <c r="A42" s="13" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Bibliography, Research Canvas and project plan</t>
+          <t>Research coordination and decision review</t>
         </is>
       </c>
       <c r="C42" s="21" t="inlineStr">
@@ -2598,175 +2526,268 @@
       </c>
       <c r="D42" s="15" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Sep 14</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
         <is>
-          <t>Sep 27</t>
+          <t>Mar 31</t>
         </is>
       </c>
       <c r="F42" s="13" t="str"/>
-      <c r="G42" s="13" t="str"/>
+      <c r="G42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="H42" s="23" t="inlineStr">
         <is>
           <t>██</t>
         </is>
       </c>
-      <c r="I42" s="13" t="str"/>
-      <c r="J42" s="13" t="str"/>
-      <c r="K42" s="13" t="str"/>
-      <c r="L42" s="13" t="str"/>
-      <c r="M42" s="13" t="str"/>
-      <c r="N42" s="13" t="str"/>
-      <c r="O42" s="13" t="str"/>
-      <c r="P42" s="13" t="str"/>
-      <c r="Q42" s="13" t="str"/>
-      <c r="R42" s="13" t="str"/>
-      <c r="S42" s="13" t="str"/>
-      <c r="T42" s="13" t="str"/>
-      <c r="U42" s="13" t="str"/>
-      <c r="V42" s="13" t="str"/>
+      <c r="I42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="S42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="T42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="U42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="V42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="W42" s="11" t="n"/>
-      <c r="X42" s="13" t="str"/>
-      <c r="Y42" s="13" t="str"/>
-      <c r="Z42" s="13" t="str"/>
+      <c r="X42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z42" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="41" customHeight="1">
       <c r="A43" s="13" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Prepare final course report, presentation and video</t>
-        </is>
-      </c>
-      <c r="C43" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Maintain and revise the living Overleaf manuscript</t>
+        </is>
+      </c>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>Nov 16</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>Dec 6</t>
+          <t>Mar 31</t>
         </is>
       </c>
       <c r="F43" s="13" t="str"/>
       <c r="G43" s="13" t="str"/>
-      <c r="H43" s="13" t="str"/>
-      <c r="I43" s="13" t="str"/>
-      <c r="J43" s="13" t="str"/>
-      <c r="K43" s="13" t="str"/>
-      <c r="L43" s="13" t="str"/>
-      <c r="M43" s="13" t="str"/>
-      <c r="N43" s="13" t="str"/>
-      <c r="O43" s="13" t="str"/>
-      <c r="P43" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q43" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="R43" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="S43" s="13" t="str"/>
-      <c r="T43" s="13" t="str"/>
-      <c r="U43" s="13" t="str"/>
-      <c r="V43" s="13" t="str"/>
+      <c r="H43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="I43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="S43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="T43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="U43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="V43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="W43" s="11" t="n"/>
-      <c r="X43" s="13" t="str"/>
-      <c r="Y43" s="13" t="str"/>
-      <c r="Z43" s="13" t="str"/>
-    </row>
-    <row r="44" ht="41" customHeight="1">
-      <c r="A44" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="B44" s="14" t="inlineStr">
-        <is>
-          <t>Course rehearsal checkpoint</t>
-        </is>
-      </c>
-      <c r="C44" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>Dec 1</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>Dec 1</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="str"/>
-      <c r="G44" s="13" t="str"/>
-      <c r="H44" s="13" t="str"/>
-      <c r="I44" s="13" t="str"/>
-      <c r="J44" s="13" t="str"/>
-      <c r="K44" s="13" t="str"/>
-      <c r="L44" s="13" t="str"/>
-      <c r="M44" s="13" t="str"/>
-      <c r="N44" s="13" t="str"/>
-      <c r="O44" s="13" t="str"/>
-      <c r="P44" s="13" t="str"/>
-      <c r="Q44" s="13" t="str"/>
-      <c r="R44" s="37" t="inlineStr">
-        <is>
-          <t>◆</t>
-        </is>
-      </c>
-      <c r="S44" s="13" t="str"/>
-      <c r="T44" s="13" t="str"/>
-      <c r="U44" s="13" t="str"/>
-      <c r="V44" s="13" t="str"/>
-      <c r="W44" s="11" t="n"/>
-      <c r="X44" s="13" t="str"/>
-      <c r="Y44" s="13" t="str"/>
-      <c r="Z44" s="13" t="str"/>
+      <c r="X43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="29" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>CAP6942 course deliverables</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="41" customHeight="1">
       <c r="A45" s="13" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>Final course report checkpoint</t>
-        </is>
-      </c>
-      <c r="C45" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Bibliography, Research Canvas and project plan</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>Dec 7</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>Dec 7</t>
+          <t>Sep 27</t>
         </is>
       </c>
       <c r="F45" s="13" t="str"/>
       <c r="G45" s="13" t="str"/>
-      <c r="H45" s="13" t="str"/>
+      <c r="H45" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="I45" s="13" t="str"/>
       <c r="J45" s="13" t="str"/>
       <c r="K45" s="13" t="str"/>
@@ -2777,11 +2798,7 @@
       <c r="P45" s="13" t="str"/>
       <c r="Q45" s="13" t="str"/>
       <c r="R45" s="13" t="str"/>
-      <c r="S45" s="37" t="inlineStr">
-        <is>
-          <t>◆</t>
-        </is>
-      </c>
+      <c r="S45" s="13" t="str"/>
       <c r="T45" s="13" t="str"/>
       <c r="U45" s="13" t="str"/>
       <c r="V45" s="13" t="str"/>
@@ -2792,11 +2809,11 @@
     </row>
     <row r="46" ht="41" customHeight="1">
       <c r="A46" s="13" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Course presentation and video checkpoint</t>
+          <t>Prepare final course report, presentation and video</t>
         </is>
       </c>
       <c r="C46" s="24" t="inlineStr">
@@ -2806,12 +2823,12 @@
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>Dec 8</t>
+          <t>Nov 16</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>Dec 8</t>
+          <t>Dec 6</t>
         </is>
       </c>
       <c r="F46" s="13" t="str"/>
@@ -2824,14 +2841,22 @@
       <c r="M46" s="13" t="str"/>
       <c r="N46" s="13" t="str"/>
       <c r="O46" s="13" t="str"/>
-      <c r="P46" s="13" t="str"/>
-      <c r="Q46" s="13" t="str"/>
-      <c r="R46" s="13" t="str"/>
-      <c r="S46" s="37" t="inlineStr">
-        <is>
-          <t>◆</t>
-        </is>
-      </c>
+      <c r="P46" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q46" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R46" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="S46" s="13" t="str"/>
       <c r="T46" s="13" t="str"/>
       <c r="U46" s="13" t="str"/>
       <c r="V46" s="13" t="str"/>
@@ -2840,35 +2865,78 @@
       <c r="Y46" s="13" t="str"/>
       <c r="Z46" s="13" t="str"/>
     </row>
-    <row r="47" ht="29" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>Research continuation</t>
-        </is>
-      </c>
+    <row r="47" ht="41" customHeight="1">
+      <c r="A47" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Course rehearsal checkpoint</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Dec 1</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>Dec 1</t>
+        </is>
+      </c>
+      <c r="F47" s="13" t="str"/>
+      <c r="G47" s="13" t="str"/>
+      <c r="H47" s="13" t="str"/>
+      <c r="I47" s="13" t="str"/>
+      <c r="J47" s="13" t="str"/>
+      <c r="K47" s="13" t="str"/>
+      <c r="L47" s="13" t="str"/>
+      <c r="M47" s="13" t="str"/>
+      <c r="N47" s="13" t="str"/>
+      <c r="O47" s="13" t="str"/>
+      <c r="P47" s="13" t="str"/>
+      <c r="Q47" s="13" t="str"/>
+      <c r="R47" s="37" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="S47" s="13" t="str"/>
+      <c r="T47" s="13" t="str"/>
+      <c r="U47" s="13" t="str"/>
+      <c r="V47" s="13" t="str"/>
+      <c r="W47" s="11" t="n"/>
+      <c r="X47" s="13" t="str"/>
+      <c r="Y47" s="13" t="str"/>
+      <c r="Z47" s="13" t="str"/>
     </row>
     <row r="48" ht="41" customHeight="1">
       <c r="A48" s="13" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Further experiments and external validation</t>
-        </is>
-      </c>
-      <c r="C48" s="29" t="inlineStr">
-        <is>
-          <t>Conditional</t>
+          <t>Final course report checkpoint</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>Jan 4</t>
+          <t>Dec 7</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>Feb 28</t>
+          <t>Dec 7</t>
         </is>
       </c>
       <c r="F48" s="13" t="str"/>
@@ -2884,30 +2952,26 @@
       <c r="P48" s="13" t="str"/>
       <c r="Q48" s="13" t="str"/>
       <c r="R48" s="13" t="str"/>
-      <c r="S48" s="13" t="str"/>
+      <c r="S48" s="37" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
       <c r="T48" s="13" t="str"/>
       <c r="U48" s="13" t="str"/>
       <c r="V48" s="13" t="str"/>
       <c r="W48" s="11" t="n"/>
-      <c r="X48" s="31" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y48" s="31" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="X48" s="13" t="str"/>
+      <c r="Y48" s="13" t="str"/>
       <c r="Z48" s="13" t="str"/>
     </row>
     <row r="49" ht="41" customHeight="1">
       <c r="A49" s="13" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Consolidate manuscript and review publication readiness</t>
+          <t>Course presentation and video checkpoint</t>
         </is>
       </c>
       <c r="C49" s="24" t="inlineStr">
@@ -2917,12 +2981,12 @@
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>Feb 1</t>
+          <t>Dec 8</t>
         </is>
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>Mar 31</t>
+          <t>Dec 8</t>
         </is>
       </c>
       <c r="F49" s="13" t="str"/>
@@ -2938,135 +3002,183 @@
       <c r="P49" s="13" t="str"/>
       <c r="Q49" s="13" t="str"/>
       <c r="R49" s="13" t="str"/>
-      <c r="S49" s="13" t="str"/>
+      <c r="S49" s="37" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
       <c r="T49" s="13" t="str"/>
       <c r="U49" s="13" t="str"/>
       <c r="V49" s="13" t="str"/>
       <c r="W49" s="11" t="n"/>
       <c r="X49" s="13" t="str"/>
-      <c r="Y49" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z49" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="41" customHeight="1">
-      <c r="A50" s="13" t="n">
+      <c r="Y49" s="13" t="str"/>
+      <c r="Z49" s="13" t="str"/>
+    </row>
+    <row r="50" ht="29" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>Research continuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="41" customHeight="1">
+      <c r="A51" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Further experiments and external validation</t>
+        </is>
+      </c>
+      <c r="C51" s="29" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>Jan 4</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>Feb 28</t>
+        </is>
+      </c>
+      <c r="F51" s="13" t="str"/>
+      <c r="G51" s="13" t="str"/>
+      <c r="H51" s="13" t="str"/>
+      <c r="I51" s="13" t="str"/>
+      <c r="J51" s="13" t="str"/>
+      <c r="K51" s="13" t="str"/>
+      <c r="L51" s="13" t="str"/>
+      <c r="M51" s="13" t="str"/>
+      <c r="N51" s="13" t="str"/>
+      <c r="O51" s="13" t="str"/>
+      <c r="P51" s="13" t="str"/>
+      <c r="Q51" s="13" t="str"/>
+      <c r="R51" s="13" t="str"/>
+      <c r="S51" s="13" t="str"/>
+      <c r="T51" s="13" t="str"/>
+      <c r="U51" s="13" t="str"/>
+      <c r="V51" s="13" t="str"/>
+      <c r="W51" s="11" t="n"/>
+      <c r="X51" s="31" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y51" s="31" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z51" s="13" t="str"/>
+    </row>
+    <row r="52" ht="41" customHeight="1">
+      <c r="A52" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Consolidate manuscript and review publication readiness</t>
+        </is>
+      </c>
+      <c r="C52" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>Feb 1</t>
+        </is>
+      </c>
+      <c r="E52" s="15" t="inlineStr">
+        <is>
+          <t>Mar 31</t>
+        </is>
+      </c>
+      <c r="F52" s="13" t="str"/>
+      <c r="G52" s="13" t="str"/>
+      <c r="H52" s="13" t="str"/>
+      <c r="I52" s="13" t="str"/>
+      <c r="J52" s="13" t="str"/>
+      <c r="K52" s="13" t="str"/>
+      <c r="L52" s="13" t="str"/>
+      <c r="M52" s="13" t="str"/>
+      <c r="N52" s="13" t="str"/>
+      <c r="O52" s="13" t="str"/>
+      <c r="P52" s="13" t="str"/>
+      <c r="Q52" s="13" t="str"/>
+      <c r="R52" s="13" t="str"/>
+      <c r="S52" s="13" t="str"/>
+      <c r="T52" s="13" t="str"/>
+      <c r="U52" s="13" t="str"/>
+      <c r="V52" s="13" t="str"/>
+      <c r="W52" s="11" t="n"/>
+      <c r="X52" s="13" t="str"/>
+      <c r="Y52" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z52" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="41" customHeight="1">
+      <c r="A53" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>March research review and next-step decision</t>
         </is>
       </c>
-      <c r="C50" s="24" t="inlineStr">
+      <c r="C53" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>Mar 31</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>Mar 31</t>
         </is>
       </c>
-      <c r="F50" s="13" t="str"/>
-      <c r="G50" s="13" t="str"/>
-      <c r="H50" s="13" t="str"/>
-      <c r="I50" s="13" t="str"/>
-      <c r="J50" s="13" t="str"/>
-      <c r="K50" s="13" t="str"/>
-      <c r="L50" s="13" t="str"/>
-      <c r="M50" s="13" t="str"/>
-      <c r="N50" s="13" t="str"/>
-      <c r="O50" s="13" t="str"/>
-      <c r="P50" s="13" t="str"/>
-      <c r="Q50" s="13" t="str"/>
-      <c r="R50" s="13" t="str"/>
-      <c r="S50" s="13" t="str"/>
-      <c r="T50" s="13" t="str"/>
-      <c r="U50" s="13" t="str"/>
-      <c r="V50" s="13" t="str"/>
-      <c r="W50" s="11" t="n"/>
-      <c r="X50" s="13" t="str"/>
-      <c r="Y50" s="13" t="str"/>
-      <c r="Z50" s="37" t="inlineStr">
+      <c r="F53" s="13" t="str"/>
+      <c r="G53" s="13" t="str"/>
+      <c r="H53" s="13" t="str"/>
+      <c r="I53" s="13" t="str"/>
+      <c r="J53" s="13" t="str"/>
+      <c r="K53" s="13" t="str"/>
+      <c r="L53" s="13" t="str"/>
+      <c r="M53" s="13" t="str"/>
+      <c r="N53" s="13" t="str"/>
+      <c r="O53" s="13" t="str"/>
+      <c r="P53" s="13" t="str"/>
+      <c r="Q53" s="13" t="str"/>
+      <c r="R53" s="13" t="str"/>
+      <c r="S53" s="13" t="str"/>
+      <c r="T53" s="13" t="str"/>
+      <c r="U53" s="13" t="str"/>
+      <c r="V53" s="13" t="str"/>
+      <c r="W53" s="11" t="n"/>
+      <c r="X53" s="13" t="str"/>
+      <c r="Y53" s="13" t="str"/>
+      <c r="Z53" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
-    </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
-      <c r="J51" s="2" t="n"/>
-      <c r="K51" s="2" t="n"/>
-      <c r="L51" s="2" t="n"/>
-      <c r="M51" s="2" t="n"/>
-      <c r="N51" s="2" t="n"/>
-      <c r="O51" s="2" t="n"/>
-      <c r="P51" s="2" t="n"/>
-      <c r="Q51" s="2" t="n"/>
-      <c r="R51" s="2" t="n"/>
-      <c r="S51" s="2" t="n"/>
-      <c r="T51" s="2" t="n"/>
-      <c r="U51" s="2" t="n"/>
-      <c r="V51" s="2" t="n"/>
-      <c r="W51" s="2" t="n"/>
-      <c r="X51" s="2" t="n"/>
-      <c r="Y51" s="2" t="n"/>
-      <c r="Z51" s="2" t="n"/>
-    </row>
-    <row r="52" ht="29" customHeight="1">
-      <c r="A52" s="33" t="inlineStr">
-        <is>
-          <t>Update the dates and corresponding week cells together. This workbook is a schedule snapshot; dates do not automatically move the bars.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
-      <c r="G53" s="2" t="n"/>
-      <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
-      <c r="J53" s="2" t="n"/>
-      <c r="K53" s="2" t="n"/>
-      <c r="L53" s="2" t="n"/>
-      <c r="M53" s="2" t="n"/>
-      <c r="N53" s="2" t="n"/>
-      <c r="O53" s="2" t="n"/>
-      <c r="P53" s="2" t="n"/>
-      <c r="Q53" s="2" t="n"/>
-      <c r="R53" s="2" t="n"/>
-      <c r="S53" s="2" t="n"/>
-      <c r="T53" s="2" t="n"/>
-      <c r="U53" s="2" t="n"/>
-      <c r="V53" s="2" t="n"/>
-      <c r="W53" s="2" t="n"/>
-      <c r="X53" s="2" t="n"/>
-      <c r="Y53" s="2" t="n"/>
-      <c r="Z53" s="2" t="n"/>
     </row>
     <row r="54" ht="24" customHeight="1">
       <c r="A54" s="2" t="n"/>
@@ -3096,43 +3208,107 @@
       <c r="Y54" s="2" t="n"/>
       <c r="Z54" s="2" t="n"/>
     </row>
-    <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="2" t="n"/>
-      <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n"/>
-      <c r="J55" s="2" t="n"/>
-      <c r="K55" s="2" t="n"/>
-      <c r="L55" s="2" t="n"/>
-      <c r="M55" s="2" t="n"/>
-      <c r="N55" s="2" t="n"/>
-      <c r="O55" s="2" t="n"/>
-      <c r="P55" s="2" t="n"/>
-      <c r="Q55" s="2" t="n"/>
-      <c r="R55" s="2" t="n"/>
-      <c r="S55" s="2" t="n"/>
-      <c r="T55" s="2" t="n"/>
-      <c r="U55" s="2" t="n"/>
-      <c r="V55" s="2" t="n"/>
-      <c r="W55" s="2" t="n"/>
-      <c r="X55" s="2" t="n"/>
-      <c r="Y55" s="2" t="n"/>
-      <c r="Z55" s="2" t="n"/>
+    <row r="55" ht="29" customHeight="1">
+      <c r="A55" s="33" t="inlineStr">
+        <is>
+          <t>Update the dates and corresponding week cells together. This workbook is a schedule snapshot; dates do not automatically move the bars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="24" customHeight="1">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="n"/>
+      <c r="N56" s="2" t="n"/>
+      <c r="O56" s="2" t="n"/>
+      <c r="P56" s="2" t="n"/>
+      <c r="Q56" s="2" t="n"/>
+      <c r="R56" s="2" t="n"/>
+      <c r="S56" s="2" t="n"/>
+      <c r="T56" s="2" t="n"/>
+      <c r="U56" s="2" t="n"/>
+      <c r="V56" s="2" t="n"/>
+      <c r="W56" s="2" t="n"/>
+      <c r="X56" s="2" t="n"/>
+      <c r="Y56" s="2" t="n"/>
+      <c r="Z56" s="2" t="n"/>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
+      <c r="M57" s="2" t="n"/>
+      <c r="N57" s="2" t="n"/>
+      <c r="O57" s="2" t="n"/>
+      <c r="P57" s="2" t="n"/>
+      <c r="Q57" s="2" t="n"/>
+      <c r="R57" s="2" t="n"/>
+      <c r="S57" s="2" t="n"/>
+      <c r="T57" s="2" t="n"/>
+      <c r="U57" s="2" t="n"/>
+      <c r="V57" s="2" t="n"/>
+      <c r="W57" s="2" t="n"/>
+      <c r="X57" s="2" t="n"/>
+      <c r="Y57" s="2" t="n"/>
+      <c r="Z57" s="2" t="n"/>
+    </row>
+    <row r="58" ht="24" customHeight="1">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
+      <c r="M58" s="2" t="n"/>
+      <c r="N58" s="2" t="n"/>
+      <c r="O58" s="2" t="n"/>
+      <c r="P58" s="2" t="n"/>
+      <c r="Q58" s="2" t="n"/>
+      <c r="R58" s="2" t="n"/>
+      <c r="S58" s="2" t="n"/>
+      <c r="T58" s="2" t="n"/>
+      <c r="U58" s="2" t="n"/>
+      <c r="V58" s="2" t="n"/>
+      <c r="W58" s="2" t="n"/>
+      <c r="X58" s="2" t="n"/>
+      <c r="Y58" s="2" t="n"/>
+      <c r="Z58" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A47:Z47"/>
     <mergeCell ref="A23:Z23"/>
+    <mergeCell ref="A44:Z44"/>
     <mergeCell ref="X5:Z5"/>
     <mergeCell ref="A3:Z3"/>
+    <mergeCell ref="A55:Z55"/>
+    <mergeCell ref="A50:Z50"/>
     <mergeCell ref="A4:Z4"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A38:Z38"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="S5:V5"/>
     <mergeCell ref="F5:I5"/>
@@ -3140,7 +3316,6 @@
     <mergeCell ref="J5:M5"/>
     <mergeCell ref="N5:R5"/>
     <mergeCell ref="A41:Z41"/>
-    <mergeCell ref="A52:Z52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3152,7 +3327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3549,12 +3724,12 @@
       </c>
       <c r="B24" s="36" t="inlineStr">
         <is>
-          <t>Run matched BioLangFusion-style comparisons</t>
+          <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (add-on 1)</t>
         </is>
       </c>
       <c r="C24" s="36" t="inlineStr">
         <is>
-          <t>Compare selected paper-inspired fusion methods and unimodal baselines on the same evaluation data, with adaptations and resources reported. Preserve null or negative results.</t>
+          <t>Compare selected paper-inspired fusion methods and unimodal baselines on the same evaluation data, with adaptations and resources reported. Widened by the research plan: reproduce BioLangFusion exactly (its encoders, codon grid, three heads, TextCNN, published splits and recipe) on Fungal, E. coli, mRNA stability, Ab1 and CoV-Vac, recording every unreported detail as a deviation; this is the matched baseline for 21. Preserve null or negative results.</t>
         </is>
       </c>
       <c r="D24" s="13" t="inlineStr">
@@ -3569,12 +3744,12 @@
       </c>
       <c r="B25" s="36" t="inlineStr">
         <is>
-          <t>Repeat diagnostics and null/control comparisons</t>
+          <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (add-on 5)</t>
         </is>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
-          <t>Check label/feature controls, synonymous-input behavior and representation diagnostics under the agreed evaluation. Test whether the claimed signal survives the relevant nulls.</t>
+          <t>Check label/feature controls, synonymous-input behavior and representation diagnostics under the agreed evaluation. Test whether the claimed signal survives the relevant nulls. Includes the mRFP synonymous control with cached embeddings: nucleotide encoders against GC3, codon-use and structure proxies; protein encoders as the invariant negative control.</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
@@ -3689,12 +3864,12 @@
       </c>
       <c r="B31" s="36" t="inlineStr">
         <is>
-          <t>Candidate additional DNA, RNA and protein encoder comparisons</t>
+          <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (add-on 2)</t>
         </is>
       </c>
       <c r="C31" s="36" t="inlineStr">
         <is>
-          <t>If selected, compare several checkpoints per modality and their combinations, including pairs within one modality, while controlling downstream capacity, input coverage and tuning. Different pretraining corpora alone do not establish complementarity. Stage 1 already covers twelve encoders, four per modality, at the representation level.</t>
+          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM, mRNA-FM, ProtBERT, ESM-2 150M, other DNA encoders), then promising triples. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2.</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -3803,72 +3978,85 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="29" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Research writing and coordination</t>
+    <row r="37" ht="58" customHeight="1">
+      <c r="A37" s="13" t="n">
+        <v>41</v>
+      </c>
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>LucaOne frozen baseline on stability and GTEx, matched comparison (add-on 3)</t>
+        </is>
+      </c>
+      <c r="C37" s="36" t="inlineStr">
+        <is>
+          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation.</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>16, 17</t>
         </is>
       </c>
     </row>
     <row r="38" ht="58" customHeight="1">
       <c r="A38" s="13" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B38" s="36" t="inlineStr">
         <is>
-          <t>Research coordination and decision review</t>
+          <t>mRNABench half-life and translation efficiency after the sequence and label gates (add-on 4)</t>
         </is>
       </c>
       <c r="C38" s="36" t="inlineStr">
         <is>
-          <t>Maintain the questions, decisions and follow-ups from regular team and advisor discussions. Confirm future meeting dates with Mina.</t>
+          <t>Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Compare CDS only, CDS + 3' UTR, full transcript, and + protein; gain over the best full-transcript baseline. Earlier if cluster time allows.</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21, 29</t>
         </is>
       </c>
     </row>
     <row r="39" ht="58" customHeight="1">
       <c r="A39" s="13" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="B39" s="36" t="inlineStr">
         <is>
-          <t>Maintain and revise the living Overleaf manuscript</t>
+          <t>Multi-teacher distillation pilot, RNA first (add-on 7)</t>
         </is>
       </c>
       <c r="C39" s="36" t="inlineStr">
         <is>
-          <t>Update methods, figures, claims, citations and open questions as research changes. Writing begins with Stage 1 and continues through review, new experiments and later consolidation.</t>
+          <t>Only after the core comparisons. Pilot one modality (RNA): distill the composition-controlled similarity structure of the teachers into one student with teacher-specific projections; evaluate on the five BioLangFusion benchmarks with the reproduced heads; report Δstudent and Δteacher with cost. Decide on three-student fusion afterwards.</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="40" ht="29" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>CAP6942 course deliverables</t>
+          <t>Research writing and coordination</t>
         </is>
       </c>
     </row>
     <row r="41" ht="58" customHeight="1">
       <c r="A41" s="13" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B41" s="36" t="inlineStr">
         <is>
-          <t>Bibliography, Research Canvas and project plan</t>
+          <t>Research coordination and decision review</t>
         </is>
       </c>
       <c r="C41" s="36" t="inlineStr">
         <is>
-          <t>Submit the annotated bibliography and Research Canvas for Team Assignment 1, and the research project plan for Team Assignment 2. Both are due September 27 at 23:59 Eastern.</t>
+          <t>Maintain the questions, decisions and follow-ups from regular team and advisor discussions. Confirm future meeting dates with Mina.</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
@@ -3879,16 +4067,16 @@
     </row>
     <row r="42" ht="58" customHeight="1">
       <c r="A42" s="13" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B42" s="36" t="inlineStr">
         <is>
-          <t>Prepare final course report, presentation and video</t>
+          <t>Maintain and revise the living Overleaf manuscript</t>
         </is>
       </c>
       <c r="C42" s="36" t="inlineStr">
         <is>
-          <t>Adapt the evolving manuscript and evidence to the course report, presentation and video requirements. Rehearse explanations and incorporate teammate and advisor feedback.</t>
+          <t>Update methods, figures, claims, citations and open questions as research changes. Writing begins with Stage 1 and continues through review, new experiments and later consolidation.</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
@@ -3897,242 +4085,262 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="58" customHeight="1">
-      <c r="A43" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="B43" s="36" t="inlineStr">
-        <is>
-          <t>Course rehearsal checkpoint</t>
-        </is>
-      </c>
-      <c r="C43" s="36" t="inlineStr">
-        <is>
-          <t>Rehearse the scientific account and record corrections; confirm the course’s exact instructions in WebCourses.</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
+    <row r="43" ht="29" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>CAP6942 course deliverables</t>
         </is>
       </c>
     </row>
     <row r="44" ht="58" customHeight="1">
       <c r="A44" s="13" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B44" s="36" t="inlineStr">
         <is>
-          <t>Final course report checkpoint</t>
+          <t>Bibliography, Research Canvas and project plan</t>
         </is>
       </c>
       <c r="C44" s="36" t="inlineStr">
         <is>
-          <t>Review evidence, attribution and AI disclosure; confirm and complete the required course submission.</t>
+          <t>Submit the annotated bibliography and Research Canvas for Team Assignment 1, and the research project plan for Team Assignment 2. Both are due September 27 at 23:59 Eastern.</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>34, 35</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="45" ht="58" customHeight="1">
       <c r="A45" s="13" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B45" s="36" t="inlineStr">
         <is>
-          <t>Course presentation and video checkpoint</t>
+          <t>Prepare final course report, presentation and video</t>
         </is>
       </c>
       <c r="C45" s="36" t="inlineStr">
         <is>
-          <t>Deliver the course presentation/video using the reviewed evidence and acknowledged limitations.</t>
+          <t>Adapt the evolving manuscript and evidence to the course report, presentation and video requirements. Rehearse explanations and incorporate teammate and advisor feedback.</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>34, 35</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="29" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>Research continuation</t>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="58" customHeight="1">
+      <c r="A46" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="B46" s="36" t="inlineStr">
+        <is>
+          <t>Course rehearsal checkpoint</t>
+        </is>
+      </c>
+      <c r="C46" s="36" t="inlineStr">
+        <is>
+          <t>Rehearse the scientific account and record corrections; confirm the course’s exact instructions in WebCourses.</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="47" ht="58" customHeight="1">
       <c r="A47" s="13" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B47" s="36" t="inlineStr">
         <is>
-          <t>Further experiments and external validation</t>
+          <t>Final course report checkpoint</t>
         </is>
       </c>
       <c r="C47" s="36" t="inlineStr">
         <is>
-          <t>Select and run extensions justified by the reviewed evidence, biological relevance, collaborators and available resources.</t>
+          <t>Review evidence, attribution and AI disclosure; confirm and complete the required course submission.</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>34, 35</t>
         </is>
       </c>
     </row>
     <row r="48" ht="58" customHeight="1">
       <c r="A48" s="13" t="n">
+        <v>37</v>
+      </c>
+      <c r="B48" s="36" t="inlineStr">
+        <is>
+          <t>Course presentation and video checkpoint</t>
+        </is>
+      </c>
+      <c r="C48" s="36" t="inlineStr">
+        <is>
+          <t>Deliver the course presentation/video using the reviewed evidence and acknowledged limitations.</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>34, 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="29" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Research continuation</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="58" customHeight="1">
+      <c r="A50" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="B50" s="36" t="inlineStr">
+        <is>
+          <t>Further experiments and external validation</t>
+        </is>
+      </c>
+      <c r="C50" s="36" t="inlineStr">
+        <is>
+          <t>Select and run extensions justified by the reviewed evidence, biological relevance, collaborators and available resources.</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="58" customHeight="1">
+      <c r="A51" s="13" t="n">
         <v>39</v>
       </c>
-      <c r="B48" s="36" t="inlineStr">
+      <c r="B51" s="36" t="inlineStr">
         <is>
           <t>Consolidate manuscript and review publication readiness</t>
         </is>
       </c>
-      <c r="C48" s="36" t="inlineStr">
+      <c r="C51" s="36" t="inlineStr">
         <is>
           <t>Refine the manuscript already underway, integrate additional evidence and seek group feedback. Venue, submission date and final research end remain undecided.</t>
         </is>
       </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="D51" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="58" customHeight="1">
-      <c r="A49" s="13" t="n">
+    <row r="52" ht="58" customHeight="1">
+      <c r="A52" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="B49" s="36" t="inlineStr">
+      <c r="B52" s="36" t="inlineStr">
         <is>
           <t>March research review and next-step decision</t>
         </is>
       </c>
-      <c r="C49" s="36" t="inlineStr">
+      <c r="C52" s="36" t="inlineStr">
         <is>
           <t>Review the evidence and decide whether to extend the experiments, revise the manuscript, prepare a submission or change direction. Adjust the timeline to the chosen next steps.</t>
         </is>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D52" s="13" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="24" customHeight="1">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-    </row>
-    <row r="51" ht="29" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+    </row>
+    <row r="54" ht="29" customHeight="1">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Planning notes</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="34" customHeight="1">
-      <c r="A52" s="33" t="inlineStr">
+    <row r="55" ht="34" customHeight="1">
+      <c r="A55" s="33" t="inlineStr">
         <is>
           <t>Update the dates and corresponding week cells together in Gantt. Keep each task ID unchanged when editing its expected output or prerequisites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="42" customHeight="1">
-      <c r="A53" s="33" t="inlineStr">
-        <is>
-          <t>The team completed the initial six-paper review by September 21. Continued interpretation and discussion run through the October 7 meeting. September 21 start dates for current work are approximate planning anchors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="42" customHeight="1">
-      <c r="A54" s="33" t="inlineStr">
-        <is>
-          <t>October 7 is the review with Mina and the target for a working alignment definition. Stage 1 includes the immediate revisions after that meeting. Future experiment dates are proposed windows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="42" customHeight="1">
-      <c r="A55" s="33" t="inlineStr">
-        <is>
-          <t>Coupled Mamba is the priority architecture comparison. Optional layer/PCA, alignment-loss, additional DNA, RNA and protein encoder comparisons and the IsoFormer fusion comparison depend on earlier findings and available capacity. The tokenizer and collaborating group must first be identified with Julian.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="33" t="inlineStr">
         <is>
-          <t>The bibliography, Research Canvas and project plan are due September 27 at 23:59 Eastern. December 1, 7 and 8 checkpoints come from the course schedule; confirm the corresponding WebCourses deadlines.</t>
+          <t>The team completed the initial six-paper review by September 21. Continued interpretation and discussion run through the October 7 meeting. September 21 start dates for current work are approximate planning anchors.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="33" t="inlineStr">
         <is>
-          <t>AI supports implementation, paper discussion, analysis and writing throughout the project. Each research task includes interpreting its evidence and revising the resulting claims. OpenAI Codex organized the original plan; Claude assisted with the September 29 revision adding the DNA modality and the October 3 status update.</t>
+          <t>October 7 is the review with Mina and the target for a working alignment definition. Stage 1 includes the immediate revisions after that meeting. Future experiment dates are proposed windows.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="33" t="inlineStr">
         <is>
+          <t>Coupled Mamba is the priority architecture comparison. Optional layer/PCA, alignment-loss, additional DNA, RNA and protein encoder comparisons and the IsoFormer fusion comparison depend on earlier findings and available capacity. The tokenizer and collaborating group must first be identified with Julian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="42" customHeight="1">
+      <c r="A59" s="33" t="inlineStr">
+        <is>
+          <t>The bibliography, Research Canvas and project plan are due September 27 at 23:59 Eastern. December 1, 7 and 8 checkpoints come from the course schedule; confirm the corresponding WebCourses deadlines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="42" customHeight="1">
+      <c r="A60" s="33" t="inlineStr">
+        <is>
+          <t>AI supports implementation, paper discussion, analysis and writing throughout the project. Each research task includes interpreting its evidence and revising the resulting claims. OpenAI Codex organized the original plan; Claude assisted with the September 29 revision adding the DNA modality and the October 3 status update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="42" customHeight="1">
+      <c r="A61" s="33" t="inlineStr">
+        <is>
           <t>Coordination began September 14. Stage 1 manuscript drafting begins September 26 and continues in Overleaf as the work develops. March is a planning horizon rather than a fixed research endpoint.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="48" customHeight="1">
-      <c r="A59" s="33" t="inlineStr">
+    <row r="62" ht="48" customHeight="1">
+      <c r="A62" s="33" t="inlineStr">
         <is>
           <t>Planning example: Mélot-Chesnel, Designing Trustworthy Generative AI Agents for Collaborative Decision Making (2026), section 4 and Figure 1, explicitly schedules reconsidering questions and hypotheses between studies. This informed retaining time for interpretation and revision. https://doi.org/10.3233/FAIA260562</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
-    </row>
-    <row r="60" ht="48" customHeight="1">
-      <c r="A60" s="33" t="inlineStr">
+    </row>
+    <row r="63" ht="48" customHeight="1">
+      <c r="A63" s="33" t="inlineStr">
         <is>
           <t>Planning example: UQ AGRC7617, Sequential mid-project assessment, uses a proposal and Gantt with supervisor discussion, followed by AI feedback on mature drafts. This illustrates review within planning. https://course-profiles.uq.edu.au/course-profiles/AGRC7617-62151-7660</t>
         </is>
       </c>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
-    </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="33" t="inlineStr">
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="33" t="inlineStr">
         <is>
           <t>These examples informed the September 27 planning discussion. They do not establish CAP6942 requirements or measured AI time savings.</t>
         </is>
       </c>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
-    </row>
-    <row r="62" ht="24" customHeight="1">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
-    </row>
-    <row r="63" ht="24" customHeight="1">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
-      <c r="D63" s="2" t="n"/>
-    </row>
-    <row r="64" ht="24" customHeight="1">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="2" t="n"/>
-      <c r="D64" s="2" t="n"/>
     </row>
     <row r="65" ht="24" customHeight="1">
       <c r="A65" s="2" t="n"/>
@@ -4146,30 +4354,48 @@
       <c r="C66" s="2" t="n"/>
       <c r="D66" s="2" t="n"/>
     </row>
+    <row r="67" ht="24" customHeight="1">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+      <c r="D67" s="2" t="n"/>
+    </row>
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+      <c r="D68" s="2" t="n"/>
+    </row>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+      <c r="D69" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A61:D61"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A53:D53"/>
     <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A62:D62"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A43:D43"/>
     <mergeCell ref="A57:D57"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A63:D63"/>
     <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A49:D49"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" ns1:id="rIdSource1" tooltip="Open planning example"/>
-    <hyperlink xmlns:ns2="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" ns2:id="rIdSource2" tooltip="Open planning example"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" tooltip="Open planning example" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" tooltip="Open planning example" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Follow Mina's research plan numbering and order; update notes, Gantt, deck, figures and links
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -255,6 +255,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -597,7 +600,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 10, 2026. Fall weeks start Monday; January to March 2027 is an adjustable monthly horizon. Rows 41 to 43 and the edits to 17, 18 and 24 fold in the research plan's add-ons.</t>
+          <t>As of October 15, 2026. Fall weeks start Monday; January to March 2027 is an adjustable monthly horizon. Rows 41 to 43 and the edits to 17, 18 and 24 fold in the research plan's seven items, under its own numbers and in its implementation order (swaps 24 before LucaOne 41).</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1652,7 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (add-on 1)</t>
+          <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (plan item 1, Phase A)</t>
         </is>
       </c>
       <c r="C25" s="24" t="inlineStr">
@@ -1703,7 +1706,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (add-on 5)</t>
+          <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (plan item 5)</t>
         </is>
       </c>
       <c r="C26" s="24" t="inlineStr">
@@ -2015,7 +2018,7 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (add-on 2)</t>
+          <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (plan item 1, Phase B)</t>
         </is>
       </c>
       <c r="C32" s="38" t="inlineStr">
@@ -2025,12 +2028,12 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Nov 9</t>
+          <t>Oct 26</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>Nov 15</t>
+          <t>Nov 8</t>
         </is>
       </c>
       <c r="F32" s="13" t="str"/>
@@ -2040,13 +2043,17 @@
       <c r="J32" s="13" t="str"/>
       <c r="K32" s="13" t="str"/>
       <c r="L32" s="13" t="str"/>
-      <c r="M32" s="13" t="str"/>
-      <c r="N32" s="13" t="str"/>
-      <c r="O32" s="39" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="M32" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N32" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O32" s="41" t="n"/>
       <c r="P32" s="13" t="str"/>
       <c r="Q32" s="13" t="str"/>
       <c r="R32" s="13" t="str"/>
@@ -2347,7 +2354,7 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>LucaOne frozen baseline on stability and GTEx, matched comparison (add-on 3)</t>
+          <t>LucaOne frozen baseline on stability and GTEx, matched comparison (plan item 2)</t>
         </is>
       </c>
       <c r="C38" s="24" t="inlineStr">
@@ -2357,12 +2364,12 @@
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>Oct 19</t>
+          <t>Nov 9</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>Nov 1</t>
+          <t>Nov 22</t>
         </is>
       </c>
       <c r="F38" s="13" t="n"/>
@@ -2371,19 +2378,19 @@
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
-      <c r="L38" s="24" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M38" s="24" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="L38" s="41" t="n"/>
+      <c r="M38" s="41" t="n"/>
       <c r="N38" s="13" t="n"/>
-      <c r="O38" s="13" t="n"/>
-      <c r="P38" s="40" t="n"/>
+      <c r="O38" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P38" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="Q38" s="40" t="n"/>
       <c r="R38" s="13" t="n"/>
       <c r="S38" s="13" t="n"/>
@@ -2401,7 +2408,7 @@
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>mRNABench half-life and translation efficiency after the sequence and label gates (add-on 4)</t>
+          <t>mRNABench half-life (plan item 3) and translation efficiency (plan item 4) after the sequence and label gates</t>
         </is>
       </c>
       <c r="C39" s="28" t="inlineStr">
@@ -2455,7 +2462,7 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Multi-teacher distillation pilot, RNA first (add-on 7)</t>
+          <t>Multi-teacher distillation, six DNA, five RNA and four protein teachers (plan item 7)</t>
         </is>
       </c>
       <c r="C40" s="28" t="inlineStr">
@@ -3724,7 +3731,7 @@
       </c>
       <c r="B24" s="36" t="inlineStr">
         <is>
-          <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (add-on 1)</t>
+          <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (plan item 1, Phase A)</t>
         </is>
       </c>
       <c r="C24" s="36" t="inlineStr">
@@ -3744,12 +3751,12 @@
       </c>
       <c r="B25" s="36" t="inlineStr">
         <is>
-          <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (add-on 5)</t>
+          <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (plan item 5)</t>
         </is>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
-          <t>Check label/feature controls, synonymous-input behavior and representation diagnostics under the agreed evaluation. Test whether the claimed signal survives the relevant nulls. Includes the mRFP synonymous control with cached embeddings: nucleotide encoders against GC3, codon-use and structure proxies; protein encoders as the invariant negative control.</t>
+          <t>Check label/feature controls, synonymous-input behavior and representation diagnostics under the agreed evaluation. Test whether the claimed signal survives the relevant nulls. Includes, in parallel, the mRFP synonymous control with cached embeddings: nucleotide encoders against GC3, codon-use and structure proxies; protein encoders as the invariant negative control.</t>
         </is>
       </c>
       <c r="D25" s="13" t="inlineStr">
@@ -3864,17 +3871,17 @@
       </c>
       <c r="B31" s="36" t="inlineStr">
         <is>
-          <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (add-on 2)</t>
+          <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (plan item 1, Phase B)</t>
         </is>
       </c>
       <c r="C31" s="36" t="inlineStr">
         <is>
-          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM, mRNA-FM, ProtBERT, ESM-2 150M, other DNA encoders), then promising triples. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2.</t>
+          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM or other suitable codon models, mRNA-FM, ProtBERT, other DNA encoders; ESM-2 150M as a further protein candidate), then promising triples, on Fungal, E. coli, mRNA stability and Ab1 (CoV-Vac if feasible). Runs directly after the reproduction (17) and before LucaOne (41), in the plan's implementation order. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2.</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17, 19</t>
         </is>
       </c>
     </row>
@@ -3984,17 +3991,17 @@
       </c>
       <c r="B37" s="36" t="inlineStr">
         <is>
-          <t>LucaOne frozen baseline on stability and GTEx, matched comparison (add-on 3)</t>
+          <t>LucaOne frozen baseline on stability and GTEx, matched comparison (plan item 2)</t>
         </is>
       </c>
       <c r="C37" s="36" t="inlineStr">
         <is>
-          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation.</t>
+          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation. After the encoder swaps (24), in the plan's implementation order.</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>16, 17</t>
+          <t>16, 17, 24</t>
         </is>
       </c>
     </row>
@@ -4004,12 +4011,12 @@
       </c>
       <c r="B38" s="36" t="inlineStr">
         <is>
-          <t>mRNABench half-life and translation efficiency after the sequence and label gates (add-on 4)</t>
+          <t>mRNABench half-life (plan item 3) and translation efficiency (plan item 4) after the sequence and label gates</t>
         </is>
       </c>
       <c r="C38" s="36" t="inlineStr">
         <is>
-          <t>Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Compare CDS only, CDS + 3' UTR, full transcript, and + protein; gain over the best full-transcript baseline. Earlier if cluster time allows.</t>
+          <t>Plan items 3 and 4, each target run separately. Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Half-life: CDS only, CDS + 3' UTR, full transcript, and + protein. Translation efficiency: 5' UTR, CDS, full transcript, + protein, and the three-encoder fusion, with RiboNN as the external benchmark. Gain over the best full-transcript baseline. Earlier if cluster time allows.</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
@@ -4024,12 +4031,12 @@
       </c>
       <c r="B39" s="36" t="inlineStr">
         <is>
-          <t>Multi-teacher distillation pilot, RNA first (add-on 7)</t>
+          <t>Multi-teacher distillation, six DNA, five RNA and four protein teachers (plan item 7)</t>
         </is>
       </c>
       <c r="C39" s="36" t="inlineStr">
         <is>
-          <t>Only after the core comparisons. Pilot one modality (RNA): distill the composition-controlled similarity structure of the teachers into one student with teacher-specific projections; evaluate on the five BioLangFusion benchmarks with the reproduced heads; report Δstudent and Δteacher with cost. Decide on three-student fusion afterwards.</t>
+          <t>Only after the core comparisons, as the research plan states. Teachers: the twelve Stage 1 encoders plus two DNA and one RNA encoder, chosen with Mina. The plan's relational objective (each teacher's cosine-similarity matrix matched through its own projection, equal weights until the uniform baseline is evaluated); RNA first as in the plan's worked example, then DNA and protein; the composition-controlled target reported beside the raw one. Evaluate each student, then fuse the three; report Δstudent and Δteacher with cost on the five BioLangFusion benchmarks with the reproduced heads.</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -4210,7 +4217,7 @@
       </c>
       <c r="C50" s="36" t="inlineStr">
         <is>
-          <t>Select and run extensions justified by the reviewed evidence, biological relevance, collaborators and available resources.</t>
+          <t>Select and run extensions justified by the reviewed evidence, biological relevance, collaborators and available resources. Includes the optional structure extension (plan item 6): sequence against sequence plus predicted structure features, only on tasks where structure plausibly acts.</t>
         </is>
       </c>
       <c r="D50" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Put Mina's research plan first: baselines and datasets before Coupled Mamba and cross-attention; resync Gantt, notes, deck, figures and READMEs
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z58"/>
+  <dimension ref="A1:Z59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -600,7 +600,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 15, 2026. Fall weeks start Monday; January to March 2027 is an adjustable monthly horizon. Rows 41 to 43 and the edits to 17, 18 and 24 fold in the research plan's seven items, under its own numbers and in its implementation order (swaps 24 before LucaOne 41).</t>
+          <t>As of October 15, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan comes first (17, 18, 24, 41, 44, 42); Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
         </is>
       </c>
     </row>
@@ -1670,35 +1670,35 @@
           <t>Oct 25</t>
         </is>
       </c>
-      <c r="F25" s="13" t="str"/>
-      <c r="G25" s="13" t="str"/>
-      <c r="H25" s="13" t="str"/>
-      <c r="I25" s="13" t="str"/>
-      <c r="J25" s="13" t="str"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="13" t="n"/>
       <c r="K25" s="37" t="inlineStr">
         <is>
           <t>██</t>
         </is>
       </c>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M25" s="13" t="str"/>
-      <c r="N25" s="13" t="str"/>
-      <c r="O25" s="13" t="str"/>
-      <c r="P25" s="13" t="str"/>
-      <c r="Q25" s="13" t="str"/>
-      <c r="R25" s="13" t="str"/>
-      <c r="S25" s="13" t="str"/>
-      <c r="T25" s="13" t="str"/>
-      <c r="U25" s="13" t="str"/>
-      <c r="V25" s="13" t="str"/>
+      <c r="L25" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="n"/>
+      <c r="N25" s="13" t="n"/>
+      <c r="O25" s="13" t="n"/>
+      <c r="P25" s="13" t="n"/>
+      <c r="Q25" s="13" t="n"/>
+      <c r="R25" s="13" t="n"/>
+      <c r="S25" s="13" t="n"/>
+      <c r="T25" s="13" t="n"/>
+      <c r="U25" s="13" t="n"/>
+      <c r="V25" s="13" t="n"/>
       <c r="W25" s="11" t="n"/>
-      <c r="X25" s="13" t="str"/>
-      <c r="Y25" s="13" t="str"/>
-      <c r="Z25" s="13" t="str"/>
+      <c r="X25" s="13" t="n"/>
+      <c r="Y25" s="13" t="n"/>
+      <c r="Z25" s="13" t="n"/>
     </row>
     <row r="26" ht="41" customHeight="1">
       <c r="A26" s="13" t="n">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Prepare Coupled Mamba inputs and feasibility tests</t>
+          <t>Prepare Coupled Mamba inputs and feasibility tests, after the research plan's baselines and datasets</t>
         </is>
       </c>
       <c r="C28" s="24" t="inlineStr">
@@ -1816,43 +1816,39 @@
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>Oct 12</t>
+          <t>Jan 4</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>Oct 25</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="str"/>
-      <c r="G28" s="13" t="str"/>
-      <c r="H28" s="13" t="str"/>
-      <c r="I28" s="13" t="str"/>
-      <c r="J28" s="13" t="str"/>
-      <c r="K28" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L28" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M28" s="13" t="str"/>
-      <c r="N28" s="13" t="str"/>
-      <c r="O28" s="13" t="str"/>
-      <c r="P28" s="13" t="str"/>
-      <c r="Q28" s="13" t="str"/>
-      <c r="R28" s="13" t="str"/>
-      <c r="S28" s="13" t="str"/>
-      <c r="T28" s="13" t="str"/>
-      <c r="U28" s="13" t="str"/>
-      <c r="V28" s="13" t="str"/>
+          <t>Jan 17</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="13" t="n"/>
+      <c r="K28" s="13" t="n"/>
+      <c r="L28" s="13" t="n"/>
+      <c r="M28" s="13" t="n"/>
+      <c r="N28" s="13" t="n"/>
+      <c r="O28" s="13" t="n"/>
+      <c r="P28" s="13" t="n"/>
+      <c r="Q28" s="13" t="n"/>
+      <c r="R28" s="13" t="n"/>
+      <c r="S28" s="13" t="n"/>
+      <c r="T28" s="13" t="n"/>
+      <c r="U28" s="13" t="n"/>
+      <c r="V28" s="13" t="n"/>
       <c r="W28" s="11" t="n"/>
-      <c r="X28" s="13" t="str"/>
-      <c r="Y28" s="13" t="str"/>
-      <c r="Z28" s="13" t="str"/>
+      <c r="X28" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y28" s="13" t="n"/>
+      <c r="Z28" s="13" t="n"/>
     </row>
     <row r="29" ht="41" customHeight="1">
       <c r="A29" s="13" t="n">
@@ -1860,7 +1856,7 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Evaluate Coupled Mamba against matched baselines</t>
+          <t>Evaluate Coupled Mamba against the research plan's baselines on its datasets</t>
         </is>
       </c>
       <c r="C29" s="24" t="inlineStr">
@@ -1870,43 +1866,43 @@
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>Oct 26</t>
+          <t>Jan 18</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>Nov 8</t>
-        </is>
-      </c>
-      <c r="F29" s="13" t="str"/>
-      <c r="G29" s="13" t="str"/>
-      <c r="H29" s="13" t="str"/>
-      <c r="I29" s="13" t="str"/>
-      <c r="J29" s="13" t="str"/>
-      <c r="K29" s="13" t="str"/>
-      <c r="L29" s="13" t="str"/>
-      <c r="M29" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N29" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O29" s="13" t="str"/>
-      <c r="P29" s="13" t="str"/>
-      <c r="Q29" s="13" t="str"/>
-      <c r="R29" s="13" t="str"/>
-      <c r="S29" s="13" t="str"/>
-      <c r="T29" s="13" t="str"/>
-      <c r="U29" s="13" t="str"/>
-      <c r="V29" s="13" t="str"/>
+          <t>Feb 7</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="13" t="n"/>
+      <c r="J29" s="13" t="n"/>
+      <c r="K29" s="13" t="n"/>
+      <c r="L29" s="13" t="n"/>
+      <c r="M29" s="13" t="n"/>
+      <c r="N29" s="13" t="n"/>
+      <c r="O29" s="13" t="n"/>
+      <c r="P29" s="13" t="n"/>
+      <c r="Q29" s="13" t="n"/>
+      <c r="R29" s="13" t="n"/>
+      <c r="S29" s="13" t="n"/>
+      <c r="T29" s="13" t="n"/>
+      <c r="U29" s="13" t="n"/>
+      <c r="V29" s="13" t="n"/>
       <c r="W29" s="11" t="n"/>
-      <c r="X29" s="13" t="str"/>
-      <c r="Y29" s="13" t="str"/>
-      <c r="Z29" s="13" t="str"/>
+      <c r="X29" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y29" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z29" s="13" t="n"/>
     </row>
     <row r="30" ht="41" customHeight="1">
       <c r="A30" s="13" t="n">
@@ -1978,39 +1974,39 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Nov 2</t>
+          <t>Feb 8</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>Nov 8</t>
-        </is>
-      </c>
-      <c r="F31" s="13" t="str"/>
-      <c r="G31" s="13" t="str"/>
-      <c r="H31" s="13" t="str"/>
-      <c r="I31" s="13" t="str"/>
-      <c r="J31" s="13" t="str"/>
-      <c r="K31" s="13" t="str"/>
-      <c r="L31" s="13" t="str"/>
-      <c r="M31" s="13" t="str"/>
-      <c r="N31" s="31" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O31" s="13" t="str"/>
-      <c r="P31" s="13" t="str"/>
-      <c r="Q31" s="13" t="str"/>
-      <c r="R31" s="13" t="str"/>
-      <c r="S31" s="13" t="str"/>
-      <c r="T31" s="13" t="str"/>
-      <c r="U31" s="13" t="str"/>
-      <c r="V31" s="13" t="str"/>
+          <t>Feb 21</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="n"/>
+      <c r="G31" s="13" t="n"/>
+      <c r="H31" s="13" t="n"/>
+      <c r="I31" s="13" t="n"/>
+      <c r="J31" s="13" t="n"/>
+      <c r="K31" s="13" t="n"/>
+      <c r="L31" s="13" t="n"/>
+      <c r="M31" s="13" t="n"/>
+      <c r="N31" s="13" t="n"/>
+      <c r="O31" s="13" t="n"/>
+      <c r="P31" s="13" t="n"/>
+      <c r="Q31" s="13" t="n"/>
+      <c r="R31" s="13" t="n"/>
+      <c r="S31" s="13" t="n"/>
+      <c r="T31" s="13" t="n"/>
+      <c r="U31" s="13" t="n"/>
+      <c r="V31" s="13" t="n"/>
       <c r="W31" s="11" t="n"/>
-      <c r="X31" s="13" t="str"/>
-      <c r="Y31" s="13" t="str"/>
-      <c r="Z31" s="13" t="str"/>
+      <c r="X31" s="13" t="n"/>
+      <c r="Y31" s="31" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z31" s="13" t="n"/>
     </row>
     <row r="32" ht="41" customHeight="1">
       <c r="A32" s="13" t="n">
@@ -2021,7 +2017,7 @@
           <t>Additional DNA, RNA and protein encoder comparison: encoder swaps in the reproduced BioLangFusion pipeline (plan item 1, Phase B)</t>
         </is>
       </c>
-      <c r="C32" s="38" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
@@ -2036,13 +2032,13 @@
           <t>Nov 8</t>
         </is>
       </c>
-      <c r="F32" s="13" t="str"/>
-      <c r="G32" s="13" t="str"/>
-      <c r="H32" s="13" t="str"/>
-      <c r="I32" s="13" t="str"/>
-      <c r="J32" s="13" t="str"/>
-      <c r="K32" s="13" t="str"/>
-      <c r="L32" s="13" t="str"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
+      <c r="L32" s="13" t="n"/>
       <c r="M32" s="37" t="inlineStr">
         <is>
           <t>██</t>
@@ -2053,18 +2049,18 @@
           <t>██</t>
         </is>
       </c>
-      <c r="O32" s="41" t="n"/>
-      <c r="P32" s="13" t="str"/>
-      <c r="Q32" s="13" t="str"/>
-      <c r="R32" s="13" t="str"/>
-      <c r="S32" s="13" t="str"/>
-      <c r="T32" s="13" t="str"/>
-      <c r="U32" s="13" t="str"/>
-      <c r="V32" s="13" t="str"/>
+      <c r="O32" s="13" t="n"/>
+      <c r="P32" s="13" t="n"/>
+      <c r="Q32" s="13" t="n"/>
+      <c r="R32" s="13" t="n"/>
+      <c r="S32" s="13" t="n"/>
+      <c r="T32" s="13" t="n"/>
+      <c r="U32" s="13" t="n"/>
+      <c r="V32" s="13" t="n"/>
       <c r="W32" s="11" t="n"/>
-      <c r="X32" s="13" t="str"/>
-      <c r="Y32" s="13" t="str"/>
-      <c r="Z32" s="13" t="str"/>
+      <c r="X32" s="13" t="n"/>
+      <c r="Y32" s="13" t="n"/>
+      <c r="Z32" s="13" t="n"/>
     </row>
     <row r="33" ht="41" customHeight="1">
       <c r="A33" s="13" t="n">
@@ -2072,49 +2068,49 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Candidate IsoFormer-style fusion comparison</t>
-        </is>
-      </c>
-      <c r="C33" s="29" t="inlineStr">
-        <is>
-          <t>Conditional</t>
+          <t>IsoFormer-style cross-attention fusion with the Stage 1 encoders, after Coupled Mamba</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>Nov 9</t>
+          <t>Feb 8</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>Nov 15</t>
-        </is>
-      </c>
-      <c r="F33" s="13" t="str"/>
-      <c r="G33" s="13" t="str"/>
-      <c r="H33" s="13" t="str"/>
-      <c r="I33" s="13" t="str"/>
-      <c r="J33" s="13" t="str"/>
-      <c r="K33" s="13" t="str"/>
-      <c r="L33" s="13" t="str"/>
-      <c r="M33" s="13" t="str"/>
-      <c r="N33" s="13" t="str"/>
-      <c r="O33" s="31" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P33" s="13" t="str"/>
-      <c r="Q33" s="13" t="str"/>
-      <c r="R33" s="13" t="str"/>
-      <c r="S33" s="13" t="str"/>
-      <c r="T33" s="13" t="str"/>
-      <c r="U33" s="13" t="str"/>
-      <c r="V33" s="13" t="str"/>
+          <t>Feb 28</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="13" t="n"/>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="13" t="n"/>
+      <c r="J33" s="13" t="n"/>
+      <c r="K33" s="13" t="n"/>
+      <c r="L33" s="13" t="n"/>
+      <c r="M33" s="13" t="n"/>
+      <c r="N33" s="13" t="n"/>
+      <c r="O33" s="13" t="n"/>
+      <c r="P33" s="13" t="n"/>
+      <c r="Q33" s="13" t="n"/>
+      <c r="R33" s="13" t="n"/>
+      <c r="S33" s="13" t="n"/>
+      <c r="T33" s="13" t="n"/>
+      <c r="U33" s="13" t="n"/>
+      <c r="V33" s="13" t="n"/>
       <c r="W33" s="11" t="n"/>
-      <c r="X33" s="13" t="str"/>
-      <c r="Y33" s="13" t="str"/>
-      <c r="Z33" s="13" t="str"/>
+      <c r="X33" s="13" t="n"/>
+      <c r="Y33" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z33" s="13" t="n"/>
     </row>
     <row r="34" ht="41" customHeight="1">
       <c r="A34" s="13" t="n">
@@ -2378,8 +2374,8 @@
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
-      <c r="L38" s="41" t="n"/>
-      <c r="M38" s="41" t="n"/>
+      <c r="L38" s="13" t="n"/>
+      <c r="M38" s="13" t="n"/>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="37" t="inlineStr">
         <is>
@@ -2391,7 +2387,7 @@
           <t>██</t>
         </is>
       </c>
-      <c r="Q38" s="40" t="n"/>
+      <c r="Q38" s="13" t="n"/>
       <c r="R38" s="13" t="n"/>
       <c r="S38" s="13" t="n"/>
       <c r="T38" s="13" t="n"/>
@@ -2411,19 +2407,19 @@
           <t>mRNABench half-life (plan item 3) and translation efficiency (plan item 4) after the sequence and label gates</t>
         </is>
       </c>
-      <c r="C39" s="28" t="inlineStr">
-        <is>
-          <t>Conditional</t>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>Jan 4</t>
+          <t>Nov 23</t>
         </is>
       </c>
       <c r="E39" s="15" t="inlineStr">
         <is>
-          <t>Feb 28</t>
+          <t>Dec 20</t>
         </is>
       </c>
       <c r="F39" s="13" t="n"/>
@@ -2436,24 +2432,32 @@
       <c r="M39" s="13" t="n"/>
       <c r="N39" s="13" t="n"/>
       <c r="O39" s="13" t="n"/>
-      <c r="P39" s="40" t="n"/>
-      <c r="Q39" s="40" t="n"/>
-      <c r="R39" s="13" t="n"/>
-      <c r="S39" s="13" t="n"/>
-      <c r="T39" s="13" t="n"/>
+      <c r="P39" s="13" t="n"/>
+      <c r="Q39" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R39" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="S39" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="T39" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="U39" s="13" t="n"/>
       <c r="V39" s="13" t="n"/>
       <c r="W39" s="11" t="n"/>
-      <c r="X39" s="28" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y39" s="28" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="X39" s="13" t="n"/>
+      <c r="Y39" s="13" t="n"/>
       <c r="Z39" s="13" t="n"/>
     </row>
     <row r="40" ht="41" customHeight="1">
@@ -2465,19 +2469,19 @@
           <t>Multi-teacher distillation, six DNA, five RNA and four protein teachers (plan item 7)</t>
         </is>
       </c>
-      <c r="C40" s="28" t="inlineStr">
+      <c r="C40" s="29" t="inlineStr">
         <is>
           <t>Conditional</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>Jan 4</t>
+          <t>Mar 1</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>Feb 28</t>
+          <t>Mar 31</t>
         </is>
       </c>
       <c r="F40" s="13" t="n"/>
@@ -2490,162 +2494,90 @@
       <c r="M40" s="13" t="n"/>
       <c r="N40" s="13" t="n"/>
       <c r="O40" s="13" t="n"/>
-      <c r="P40" s="40" t="n"/>
-      <c r="Q40" s="40" t="n"/>
+      <c r="P40" s="13" t="n"/>
+      <c r="Q40" s="13" t="n"/>
       <c r="R40" s="13" t="n"/>
       <c r="S40" s="13" t="n"/>
       <c r="T40" s="13" t="n"/>
       <c r="U40" s="13" t="n"/>
       <c r="V40" s="13" t="n"/>
       <c r="W40" s="11" t="n"/>
-      <c r="X40" s="28" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y40" s="28" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z40" s="13" t="n"/>
-    </row>
-    <row r="41" ht="29" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="X40" s="13" t="n"/>
+      <c r="Y40" s="13" t="n"/>
+      <c r="Z40" s="31" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="41" customHeight="1">
+      <c r="A41" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>IsoFormer's cross-attention aggregator reproduced on GTEx as a baseline, beside LucaOne (not on the plan's list)</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Nov 9</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>Nov 22</t>
+        </is>
+      </c>
+      <c r="F41" s="13" t="n"/>
+      <c r="G41" s="13" t="n"/>
+      <c r="H41" s="13" t="n"/>
+      <c r="I41" s="13" t="n"/>
+      <c r="J41" s="13" t="n"/>
+      <c r="K41" s="13" t="n"/>
+      <c r="L41" s="13" t="n"/>
+      <c r="M41" s="13" t="n"/>
+      <c r="N41" s="13" t="n"/>
+      <c r="O41" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P41" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q41" s="13" t="n"/>
+      <c r="R41" s="13" t="n"/>
+      <c r="S41" s="13" t="n"/>
+      <c r="T41" s="13" t="n"/>
+      <c r="U41" s="13" t="n"/>
+      <c r="V41" s="13" t="n"/>
+      <c r="W41" s="11" t="n"/>
+      <c r="X41" s="13" t="n"/>
+      <c r="Y41" s="13" t="n"/>
+      <c r="Z41" s="13" t="n"/>
+    </row>
+    <row r="42" ht="29" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Research writing and coordination</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="41" customHeight="1">
-      <c r="A42" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>Research coordination and decision review</t>
-        </is>
-      </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>Sep 14</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>Mar 31</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="str"/>
-      <c r="G42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="H42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="J42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="K42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="R42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="S42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="T42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="U42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="V42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="W42" s="11" t="n"/>
-      <c r="X42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z42" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
         </is>
       </c>
     </row>
     <row r="43" ht="41" customHeight="1">
       <c r="A43" s="13" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Maintain and revise the living Overleaf manuscript</t>
+          <t>Research coordination and decision review</t>
         </is>
       </c>
       <c r="C43" s="21" t="inlineStr">
@@ -2655,7 +2587,7 @@
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Sep 14</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
@@ -2664,7 +2596,11 @@
         </is>
       </c>
       <c r="F43" s="13" t="str"/>
-      <c r="G43" s="13" t="str"/>
+      <c r="G43" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="H43" s="23" t="inlineStr">
         <is>
           <t>██</t>
@@ -2757,90 +2693,162 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="29" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="44" ht="41" customHeight="1">
+      <c r="A44" s="13" t="n">
+        <v>32</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Maintain and revise the living Overleaf manuscript</t>
+        </is>
+      </c>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>Mar 31</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="str"/>
+      <c r="G44" s="13" t="str"/>
+      <c r="H44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="I44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="K44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="S44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="T44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="U44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="V44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="W44" s="11" t="n"/>
+      <c r="X44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Y44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Z44" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="29" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>CAP6942 course deliverables</t>
         </is>
       </c>
-    </row>
-    <row r="45" ht="41" customHeight="1">
-      <c r="A45" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>Bibliography, Research Canvas and project plan</t>
-        </is>
-      </c>
-      <c r="C45" s="21" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="D45" s="15" t="inlineStr">
-        <is>
-          <t>Sep 26</t>
-        </is>
-      </c>
-      <c r="E45" s="15" t="inlineStr">
-        <is>
-          <t>Sep 27</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="str"/>
-      <c r="G45" s="13" t="str"/>
-      <c r="H45" s="23" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I45" s="13" t="str"/>
-      <c r="J45" s="13" t="str"/>
-      <c r="K45" s="13" t="str"/>
-      <c r="L45" s="13" t="str"/>
-      <c r="M45" s="13" t="str"/>
-      <c r="N45" s="13" t="str"/>
-      <c r="O45" s="13" t="str"/>
-      <c r="P45" s="13" t="str"/>
-      <c r="Q45" s="13" t="str"/>
-      <c r="R45" s="13" t="str"/>
-      <c r="S45" s="13" t="str"/>
-      <c r="T45" s="13" t="str"/>
-      <c r="U45" s="13" t="str"/>
-      <c r="V45" s="13" t="str"/>
-      <c r="W45" s="11" t="n"/>
-      <c r="X45" s="13" t="str"/>
-      <c r="Y45" s="13" t="str"/>
-      <c r="Z45" s="13" t="str"/>
     </row>
     <row r="46" ht="41" customHeight="1">
       <c r="A46" s="13" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Prepare final course report, presentation and video</t>
-        </is>
-      </c>
-      <c r="C46" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Bibliography, Research Canvas and project plan</t>
+        </is>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>Nov 16</t>
+          <t>Sep 26</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>Dec 6</t>
+          <t>Sep 27</t>
         </is>
       </c>
       <c r="F46" s="13" t="str"/>
       <c r="G46" s="13" t="str"/>
-      <c r="H46" s="13" t="str"/>
+      <c r="H46" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="I46" s="13" t="str"/>
       <c r="J46" s="13" t="str"/>
       <c r="K46" s="13" t="str"/>
@@ -2848,21 +2856,9 @@
       <c r="M46" s="13" t="str"/>
       <c r="N46" s="13" t="str"/>
       <c r="O46" s="13" t="str"/>
-      <c r="P46" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Q46" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="R46" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="P46" s="13" t="str"/>
+      <c r="Q46" s="13" t="str"/>
+      <c r="R46" s="13" t="str"/>
       <c r="S46" s="13" t="str"/>
       <c r="T46" s="13" t="str"/>
       <c r="U46" s="13" t="str"/>
@@ -2874,11 +2870,11 @@
     </row>
     <row r="47" ht="41" customHeight="1">
       <c r="A47" s="13" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Course rehearsal checkpoint</t>
+          <t>Prepare final course report, presentation and video</t>
         </is>
       </c>
       <c r="C47" s="24" t="inlineStr">
@@ -2888,12 +2884,12 @@
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>Dec 1</t>
+          <t>Nov 16</t>
         </is>
       </c>
       <c r="E47" s="15" t="inlineStr">
         <is>
-          <t>Dec 1</t>
+          <t>Dec 6</t>
         </is>
       </c>
       <c r="F47" s="13" t="str"/>
@@ -2906,11 +2902,19 @@
       <c r="M47" s="13" t="str"/>
       <c r="N47" s="13" t="str"/>
       <c r="O47" s="13" t="str"/>
-      <c r="P47" s="13" t="str"/>
-      <c r="Q47" s="13" t="str"/>
+      <c r="P47" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q47" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="R47" s="37" t="inlineStr">
         <is>
-          <t>◆</t>
+          <t>██</t>
         </is>
       </c>
       <c r="S47" s="13" t="str"/>
@@ -2924,11 +2928,11 @@
     </row>
     <row r="48" ht="41" customHeight="1">
       <c r="A48" s="13" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Final course report checkpoint</t>
+          <t>Course rehearsal checkpoint</t>
         </is>
       </c>
       <c r="C48" s="24" t="inlineStr">
@@ -2938,12 +2942,12 @@
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>Dec 7</t>
+          <t>Dec 1</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>Dec 7</t>
+          <t>Dec 1</t>
         </is>
       </c>
       <c r="F48" s="13" t="str"/>
@@ -2958,12 +2962,12 @@
       <c r="O48" s="13" t="str"/>
       <c r="P48" s="13" t="str"/>
       <c r="Q48" s="13" t="str"/>
-      <c r="R48" s="13" t="str"/>
-      <c r="S48" s="37" t="inlineStr">
+      <c r="R48" s="37" t="inlineStr">
         <is>
           <t>◆</t>
         </is>
       </c>
+      <c r="S48" s="13" t="str"/>
       <c r="T48" s="13" t="str"/>
       <c r="U48" s="13" t="str"/>
       <c r="V48" s="13" t="str"/>
@@ -2974,11 +2978,11 @@
     </row>
     <row r="49" ht="41" customHeight="1">
       <c r="A49" s="13" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Course presentation and video checkpoint</t>
+          <t>Final course report checkpoint</t>
         </is>
       </c>
       <c r="C49" s="24" t="inlineStr">
@@ -2988,12 +2992,12 @@
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>Dec 8</t>
+          <t>Dec 7</t>
         </is>
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>Dec 8</t>
+          <t>Dec 7</t>
         </is>
       </c>
       <c r="F49" s="13" t="str"/>
@@ -3022,84 +3026,80 @@
       <c r="Y49" s="13" t="str"/>
       <c r="Z49" s="13" t="str"/>
     </row>
-    <row r="50" ht="29" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="50" ht="41" customHeight="1">
+      <c r="A50" s="13" t="n">
+        <v>37</v>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Course presentation and video checkpoint</t>
+        </is>
+      </c>
+      <c r="C50" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>Dec 8</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>Dec 8</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="str"/>
+      <c r="G50" s="13" t="str"/>
+      <c r="H50" s="13" t="str"/>
+      <c r="I50" s="13" t="str"/>
+      <c r="J50" s="13" t="str"/>
+      <c r="K50" s="13" t="str"/>
+      <c r="L50" s="13" t="str"/>
+      <c r="M50" s="13" t="str"/>
+      <c r="N50" s="13" t="str"/>
+      <c r="O50" s="13" t="str"/>
+      <c r="P50" s="13" t="str"/>
+      <c r="Q50" s="13" t="str"/>
+      <c r="R50" s="13" t="str"/>
+      <c r="S50" s="37" t="inlineStr">
+        <is>
+          <t>◆</t>
+        </is>
+      </c>
+      <c r="T50" s="13" t="str"/>
+      <c r="U50" s="13" t="str"/>
+      <c r="V50" s="13" t="str"/>
+      <c r="W50" s="11" t="n"/>
+      <c r="X50" s="13" t="str"/>
+      <c r="Y50" s="13" t="str"/>
+      <c r="Z50" s="13" t="str"/>
+    </row>
+    <row r="51" ht="29" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>Research continuation</t>
         </is>
       </c>
-    </row>
-    <row r="51" ht="41" customHeight="1">
-      <c r="A51" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="B51" s="14" t="inlineStr">
-        <is>
-          <t>Further experiments and external validation</t>
-        </is>
-      </c>
-      <c r="C51" s="29" t="inlineStr">
-        <is>
-          <t>Conditional</t>
-        </is>
-      </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>Jan 4</t>
-        </is>
-      </c>
-      <c r="E51" s="15" t="inlineStr">
-        <is>
-          <t>Feb 28</t>
-        </is>
-      </c>
-      <c r="F51" s="13" t="str"/>
-      <c r="G51" s="13" t="str"/>
-      <c r="H51" s="13" t="str"/>
-      <c r="I51" s="13" t="str"/>
-      <c r="J51" s="13" t="str"/>
-      <c r="K51" s="13" t="str"/>
-      <c r="L51" s="13" t="str"/>
-      <c r="M51" s="13" t="str"/>
-      <c r="N51" s="13" t="str"/>
-      <c r="O51" s="13" t="str"/>
-      <c r="P51" s="13" t="str"/>
-      <c r="Q51" s="13" t="str"/>
-      <c r="R51" s="13" t="str"/>
-      <c r="S51" s="13" t="str"/>
-      <c r="T51" s="13" t="str"/>
-      <c r="U51" s="13" t="str"/>
-      <c r="V51" s="13" t="str"/>
-      <c r="W51" s="11" t="n"/>
-      <c r="X51" s="31" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Y51" s="31" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z51" s="13" t="str"/>
     </row>
     <row r="52" ht="41" customHeight="1">
       <c r="A52" s="13" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Consolidate manuscript and review publication readiness</t>
-        </is>
-      </c>
-      <c r="C52" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Further experiments and external validation</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>Conditional</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>Feb 1</t>
+          <t>Mar 1</t>
         </is>
       </c>
       <c r="E52" s="15" t="inlineStr">
@@ -3107,31 +3107,27 @@
           <t>Mar 31</t>
         </is>
       </c>
-      <c r="F52" s="13" t="str"/>
-      <c r="G52" s="13" t="str"/>
-      <c r="H52" s="13" t="str"/>
-      <c r="I52" s="13" t="str"/>
-      <c r="J52" s="13" t="str"/>
-      <c r="K52" s="13" t="str"/>
-      <c r="L52" s="13" t="str"/>
-      <c r="M52" s="13" t="str"/>
-      <c r="N52" s="13" t="str"/>
-      <c r="O52" s="13" t="str"/>
-      <c r="P52" s="13" t="str"/>
-      <c r="Q52" s="13" t="str"/>
-      <c r="R52" s="13" t="str"/>
-      <c r="S52" s="13" t="str"/>
-      <c r="T52" s="13" t="str"/>
-      <c r="U52" s="13" t="str"/>
-      <c r="V52" s="13" t="str"/>
+      <c r="F52" s="13" t="n"/>
+      <c r="G52" s="13" t="n"/>
+      <c r="H52" s="13" t="n"/>
+      <c r="I52" s="13" t="n"/>
+      <c r="J52" s="13" t="n"/>
+      <c r="K52" s="13" t="n"/>
+      <c r="L52" s="13" t="n"/>
+      <c r="M52" s="13" t="n"/>
+      <c r="N52" s="13" t="n"/>
+      <c r="O52" s="13" t="n"/>
+      <c r="P52" s="13" t="n"/>
+      <c r="Q52" s="13" t="n"/>
+      <c r="R52" s="13" t="n"/>
+      <c r="S52" s="13" t="n"/>
+      <c r="T52" s="13" t="n"/>
+      <c r="U52" s="13" t="n"/>
+      <c r="V52" s="13" t="n"/>
       <c r="W52" s="11" t="n"/>
-      <c r="X52" s="13" t="str"/>
-      <c r="Y52" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="Z52" s="37" t="inlineStr">
+      <c r="X52" s="13" t="n"/>
+      <c r="Y52" s="13" t="n"/>
+      <c r="Z52" s="31" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -3139,11 +3135,11 @@
     </row>
     <row r="53" ht="41" customHeight="1">
       <c r="A53" s="13" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>March research review and next-step decision</t>
+          <t>Consolidate manuscript and review publication readiness</t>
         </is>
       </c>
       <c r="C53" s="24" t="inlineStr">
@@ -3153,7 +3149,7 @@
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>Mar 31</t>
+          <t>Feb 1</t>
         </is>
       </c>
       <c r="E53" s="15" t="inlineStr">
@@ -3180,75 +3176,101 @@
       <c r="V53" s="13" t="str"/>
       <c r="W53" s="11" t="n"/>
       <c r="X53" s="13" t="str"/>
-      <c r="Y53" s="13" t="str"/>
+      <c r="Y53" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="Z53" s="37" t="inlineStr">
         <is>
+          <t>██</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="41" customHeight="1">
+      <c r="A54" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>March research review and next-step decision</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>Mar 31</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>Mar 31</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="str"/>
+      <c r="G54" s="13" t="str"/>
+      <c r="H54" s="13" t="str"/>
+      <c r="I54" s="13" t="str"/>
+      <c r="J54" s="13" t="str"/>
+      <c r="K54" s="13" t="str"/>
+      <c r="L54" s="13" t="str"/>
+      <c r="M54" s="13" t="str"/>
+      <c r="N54" s="13" t="str"/>
+      <c r="O54" s="13" t="str"/>
+      <c r="P54" s="13" t="str"/>
+      <c r="Q54" s="13" t="str"/>
+      <c r="R54" s="13" t="str"/>
+      <c r="S54" s="13" t="str"/>
+      <c r="T54" s="13" t="str"/>
+      <c r="U54" s="13" t="str"/>
+      <c r="V54" s="13" t="str"/>
+      <c r="W54" s="11" t="n"/>
+      <c r="X54" s="13" t="str"/>
+      <c r="Y54" s="13" t="str"/>
+      <c r="Z54" s="37" t="inlineStr">
+        <is>
           <t>◆</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="24" customHeight="1">
-      <c r="A54" s="2" t="n"/>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
-      <c r="J54" s="2" t="n"/>
-      <c r="K54" s="2" t="n"/>
-      <c r="L54" s="2" t="n"/>
-      <c r="M54" s="2" t="n"/>
-      <c r="N54" s="2" t="n"/>
-      <c r="O54" s="2" t="n"/>
-      <c r="P54" s="2" t="n"/>
-      <c r="Q54" s="2" t="n"/>
-      <c r="R54" s="2" t="n"/>
-      <c r="S54" s="2" t="n"/>
-      <c r="T54" s="2" t="n"/>
-      <c r="U54" s="2" t="n"/>
-      <c r="V54" s="2" t="n"/>
-      <c r="W54" s="2" t="n"/>
-      <c r="X54" s="2" t="n"/>
-      <c r="Y54" s="2" t="n"/>
-      <c r="Z54" s="2" t="n"/>
-    </row>
-    <row r="55" ht="29" customHeight="1">
-      <c r="A55" s="33" t="inlineStr">
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="n"/>
+      <c r="M55" s="2" t="n"/>
+      <c r="N55" s="2" t="n"/>
+      <c r="O55" s="2" t="n"/>
+      <c r="P55" s="2" t="n"/>
+      <c r="Q55" s="2" t="n"/>
+      <c r="R55" s="2" t="n"/>
+      <c r="S55" s="2" t="n"/>
+      <c r="T55" s="2" t="n"/>
+      <c r="U55" s="2" t="n"/>
+      <c r="V55" s="2" t="n"/>
+      <c r="W55" s="2" t="n"/>
+      <c r="X55" s="2" t="n"/>
+      <c r="Y55" s="2" t="n"/>
+      <c r="Z55" s="2" t="n"/>
+    </row>
+    <row r="56" ht="29" customHeight="1">
+      <c r="A56" s="33" t="inlineStr">
         <is>
           <t>Update the dates and corresponding week cells together. This workbook is a schedule snapshot; dates do not automatically move the bars.</t>
         </is>
       </c>
-    </row>
-    <row r="56" ht="24" customHeight="1">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="2" t="n"/>
-      <c r="J56" s="2" t="n"/>
-      <c r="K56" s="2" t="n"/>
-      <c r="L56" s="2" t="n"/>
-      <c r="M56" s="2" t="n"/>
-      <c r="N56" s="2" t="n"/>
-      <c r="O56" s="2" t="n"/>
-      <c r="P56" s="2" t="n"/>
-      <c r="Q56" s="2" t="n"/>
-      <c r="R56" s="2" t="n"/>
-      <c r="S56" s="2" t="n"/>
-      <c r="T56" s="2" t="n"/>
-      <c r="U56" s="2" t="n"/>
-      <c r="V56" s="2" t="n"/>
-      <c r="W56" s="2" t="n"/>
-      <c r="X56" s="2" t="n"/>
-      <c r="Y56" s="2" t="n"/>
-      <c r="Z56" s="2" t="n"/>
     </row>
     <row r="57" ht="24" customHeight="1">
       <c r="A57" s="2" t="n"/>
@@ -3306,14 +3328,42 @@
       <c r="Y58" s="2" t="n"/>
       <c r="Z58" s="2" t="n"/>
     </row>
+    <row r="59" ht="24" customHeight="1">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
+      <c r="M59" s="2" t="n"/>
+      <c r="N59" s="2" t="n"/>
+      <c r="O59" s="2" t="n"/>
+      <c r="P59" s="2" t="n"/>
+      <c r="Q59" s="2" t="n"/>
+      <c r="R59" s="2" t="n"/>
+      <c r="S59" s="2" t="n"/>
+      <c r="T59" s="2" t="n"/>
+      <c r="U59" s="2" t="n"/>
+      <c r="V59" s="2" t="n"/>
+      <c r="W59" s="2" t="n"/>
+      <c r="X59" s="2" t="n"/>
+      <c r="Y59" s="2" t="n"/>
+      <c r="Z59" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A23:Z23"/>
-    <mergeCell ref="A44:Z44"/>
+    <mergeCell ref="A45:Z45"/>
     <mergeCell ref="X5:Z5"/>
     <mergeCell ref="A3:Z3"/>
-    <mergeCell ref="A55:Z55"/>
-    <mergeCell ref="A50:Z50"/>
+    <mergeCell ref="A56:Z56"/>
+    <mergeCell ref="A51:Z51"/>
     <mergeCell ref="A4:Z4"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A2:Z2"/>
@@ -3322,7 +3372,7 @@
     <mergeCell ref="A7:Z7"/>
     <mergeCell ref="J5:M5"/>
     <mergeCell ref="N5:R5"/>
-    <mergeCell ref="A41:Z41"/>
+    <mergeCell ref="A42:Z42"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3334,7 +3384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3689,7 +3739,7 @@
       </c>
       <c r="C21" s="36" t="inlineStr">
         <is>
-          <t>Set biological question, target, evaluation unit, data exclusions, checkpoints, preprocessing, metrics, seeds, tuning budget and success/stop criteria. Architecture priority remains Coupled Mamba; details follow the review.</t>
+          <t>Set biological question, target, evaluation unit, data exclusions, checkpoints, preprocessing, metrics, seeds, tuning budget and success/stop criteria. The research plan's baselines come first; Coupled Mamba remains the project's first design after them. Details follow the review.</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -3791,17 +3841,17 @@
       </c>
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>Prepare Coupled Mamba inputs and feasibility tests</t>
+          <t>Prepare Coupled Mamba inputs and feasibility tests, after the research plan's baselines and datasets</t>
         </is>
       </c>
       <c r="C27" s="36" t="inlineStr">
         <is>
-          <t>Implement the prioritized architecture with explicit sequence/feature correspondence; test dimensions, controlled cases and resource feasibility while baseline analysis proceeds.</t>
+          <t>Implement the project's first design with explicit sequence/feature correspondence; test dimensions, controlled cases and resource feasibility once the research plan's baselines (17, 24, 41, 44) and datasets (42) are in place.</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>15, 16</t>
+          <t>17, 24, 41, 42, 44</t>
         </is>
       </c>
     </row>
@@ -3811,17 +3861,17 @@
       </c>
       <c r="B28" s="36" t="inlineStr">
         <is>
-          <t>Evaluate Coupled Mamba against matched baselines</t>
+          <t>Evaluate Coupled Mamba against the research plan's baselines on its datasets</t>
         </is>
       </c>
       <c r="C28" s="36" t="inlineStr">
         <is>
-          <t>Compare predictive performance, uncertainty, runtime and memory under the matched evaluation protocol. Interpret gains, losses or unchanged performance against the baseline.</t>
+          <t>Compare predictive performance, uncertainty, runtime and memory under the matched evaluation protocol. Score it against every research plan baseline (reproduced heads, encoder swaps, LucaOne, IsoFormer) on every dataset of the plan, including half-life and translation efficiency (42). Interpret gains, losses or unchanged performance.</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>19, 20</t>
+          <t>19, 20, 24, 41, 42, 44</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3911,7 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>19, 20</t>
+          <t>21</t>
         </is>
       </c>
     </row>
@@ -3891,17 +3941,17 @@
       </c>
       <c r="B32" s="36" t="inlineStr">
         <is>
-          <t>Candidate IsoFormer-style fusion comparison</t>
+          <t>IsoFormer-style cross-attention fusion with the Stage 1 encoders, after Coupled Mamba</t>
         </is>
       </c>
       <c r="C32" s="36" t="inlineStr">
         <is>
-          <t>Evaluate the second-priority cross-attention candidate only if the reviewed research question and resource budget justify it. Report relevant differences from IsoFormer’s fine-tuning regime.</t>
+          <t>The project's second design, after Coupled Mamba: cross-attention with the encoders Stage 1 points to, on GTEx and as the competitor on coding sequence, scored against the same baselines, including IsoFormer's own aggregator (44). Report relevant differences from IsoFormer’s fine-tuning regime.</t>
         </is>
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>21, 44</t>
         </is>
       </c>
     </row>
@@ -3981,7 +4031,7 @@
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>19, 21</t>
+          <t>19, 24, 41, 44</t>
         </is>
       </c>
     </row>
@@ -4005,7 +4055,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="58" customHeight="1">
+    <row r="38" ht="72" customHeight="1">
       <c r="A38" s="13" t="n">
         <v>42</v>
       </c>
@@ -4016,16 +4066,16 @@
       </c>
       <c r="C38" s="36" t="inlineStr">
         <is>
-          <t>Plan items 3 and 4, each target run separately. Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Half-life: CDS only, CDS + 3' UTR, full transcript, and + protein. Translation efficiency: 5' UTR, CDS, full transcript, + protein, and the three-encoder fusion, with RiboNN as the external benchmark. Gain over the best full-transcript baseline. Earlier if cluster time allows.</t>
+          <t>Plan items 3 and 4, each target run separately. Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Half-life: CDS only, CDS + 3' UTR, full transcript, and + protein. Translation efficiency: 5' UTR, CDS, full transcript, + protein, and the three-encoder fusion, with RiboNN as the external benchmark. Gain over the best full-transcript baseline. After the plan's baselines (24, 41, 44) and before the project's designs (20, 21), so every baseline is scored on these tasks.</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>21, 29</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="58" customHeight="1">
+          <t>17, 24, 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
       <c r="A39" s="13" t="n">
         <v>43</v>
       </c>
@@ -4036,101 +4086,101 @@
       </c>
       <c r="C39" s="36" t="inlineStr">
         <is>
-          <t>Only after the core comparisons, as the research plan states. Teachers: the twelve Stage 1 encoders plus two DNA and one RNA encoder, chosen with Mina. The plan's relational objective (each teacher's cosine-similarity matrix matched through its own projection, equal weights until the uniform baseline is evaluated); RNA first as in the plan's worked example, then DNA and protein; the composition-controlled target reported beside the raw one. Evaluate each student, then fuse the three; report Δstudent and Δteacher with cost on the five BioLangFusion benchmarks with the reproduced heads.</t>
+          <t>In March, after the core comparisons and the project's designs, as the research plan states. Teachers: the twelve Stage 1 encoders plus two DNA and one RNA encoder, chosen with Mina. The plan's relational objective (each teacher's cosine-similarity matrix matched through its own projection, equal weights until the uniform baseline is evaluated); RNA first as in the plan's worked example, then DNA and protein; the composition-controlled target reported beside the raw one. Evaluate each student, then fuse the three; report Δstudent and Δteacher with cost on the five BioLangFusion benchmarks with the reproduced heads.</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
         <is>
-          <t>29</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="29" customHeight="1">
-      <c r="A40" s="8" t="inlineStr">
+          <t>21, 25, 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="58" customHeight="1">
+      <c r="A40" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="B40" s="36" t="inlineStr">
+        <is>
+          <t>IsoFormer's cross-attention aggregator reproduced on GTEx as a baseline, beside LucaOne (not on the plan's list)</t>
+        </is>
+      </c>
+      <c r="C40" s="36" t="inlineStr">
+        <is>
+          <t>Not on the research plan's list, but the published distinct-molecule baseline: IsoFormer's cross-attention aggregator with frozen Nucleotide Transformer v2 (DNA window), each RNA encoder in the transcript role and ESM-2 150M (protein), on the GTEx pilot and then the full table; R² and Spearman averaged over tissues as IsoFormer reports them, with the four length features beside it. Runs beside LucaOne (41), before the project's designs.</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>8, 9, 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="29" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>Research writing and coordination</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="58" customHeight="1">
-      <c r="A41" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="B41" s="36" t="inlineStr">
-        <is>
-          <t>Research coordination and decision review</t>
-        </is>
-      </c>
-      <c r="C41" s="36" t="inlineStr">
-        <is>
-          <t>Maintain the questions, decisions and follow-ups from regular team and advisor discussions. Confirm future meeting dates with Mina.</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
     <row r="42" ht="58" customHeight="1">
       <c r="A42" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="B42" s="36" t="inlineStr">
+        <is>
+          <t>Research coordination and decision review</t>
+        </is>
+      </c>
+      <c r="C42" s="36" t="inlineStr">
+        <is>
+          <t>Maintain the questions, decisions and follow-ups from regular team and advisor discussions. Confirm future meeting dates with Mina.</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="58" customHeight="1">
+      <c r="A43" s="13" t="n">
         <v>32</v>
       </c>
-      <c r="B42" s="36" t="inlineStr">
+      <c r="B43" s="36" t="inlineStr">
         <is>
           <t>Maintain and revise the living Overleaf manuscript</t>
         </is>
       </c>
-      <c r="C42" s="36" t="inlineStr">
+      <c r="C43" s="36" t="inlineStr">
         <is>
           <t>Update methods, figures, claims, citations and open questions as research changes. Writing begins with Stage 1 and continues through review, new experiments and later consolidation.</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="29" customHeight="1">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="44" ht="29" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>CAP6942 course deliverables</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="58" customHeight="1">
-      <c r="A44" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="B44" s="36" t="inlineStr">
-        <is>
-          <t>Bibliography, Research Canvas and project plan</t>
-        </is>
-      </c>
-      <c r="C44" s="36" t="inlineStr">
-        <is>
-          <t>Submit the annotated bibliography and Research Canvas for Team Assignment 1, and the research project plan for Team Assignment 2. Both are due September 27 at 23:59 Eastern.</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
     </row>
     <row r="45" ht="58" customHeight="1">
       <c r="A45" s="13" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B45" s="36" t="inlineStr">
         <is>
-          <t>Prepare final course report, presentation and video</t>
+          <t>Bibliography, Research Canvas and project plan</t>
         </is>
       </c>
       <c r="C45" s="36" t="inlineStr">
         <is>
-          <t>Adapt the evolving manuscript and evidence to the course report, presentation and video requirements. Rehearse explanations and incorporate teammate and advisor feedback.</t>
+          <t>Submit the annotated bibliography and Research Canvas for Team Assignment 1, and the research project plan for Team Assignment 2. Both are due September 27 at 23:59 Eastern.</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
@@ -4141,16 +4191,16 @@
     </row>
     <row r="46" ht="58" customHeight="1">
       <c r="A46" s="13" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B46" s="36" t="inlineStr">
         <is>
-          <t>Course rehearsal checkpoint</t>
+          <t>Prepare final course report, presentation and video</t>
         </is>
       </c>
       <c r="C46" s="36" t="inlineStr">
         <is>
-          <t>Rehearse the scientific account and record corrections; confirm the course’s exact instructions in WebCourses.</t>
+          <t>Adapt the evolving manuscript and evidence to the course report, presentation and video requirements. Rehearse explanations and incorporate teammate and advisor feedback.</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
@@ -4161,199 +4211,213 @@
     </row>
     <row r="47" ht="58" customHeight="1">
       <c r="A47" s="13" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B47" s="36" t="inlineStr">
         <is>
-          <t>Final course report checkpoint</t>
+          <t>Course rehearsal checkpoint</t>
         </is>
       </c>
       <c r="C47" s="36" t="inlineStr">
         <is>
-          <t>Review evidence, attribution and AI disclosure; confirm and complete the required course submission.</t>
+          <t>Rehearse the scientific account and record corrections; confirm the course’s exact instructions in WebCourses.</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>34, 35</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="48" ht="58" customHeight="1">
       <c r="A48" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="B48" s="36" t="inlineStr">
+        <is>
+          <t>Final course report checkpoint</t>
+        </is>
+      </c>
+      <c r="C48" s="36" t="inlineStr">
+        <is>
+          <t>Review evidence, attribution and AI disclosure; confirm and complete the required course submission.</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>34, 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="58" customHeight="1">
+      <c r="A49" s="13" t="n">
         <v>37</v>
       </c>
-      <c r="B48" s="36" t="inlineStr">
+      <c r="B49" s="36" t="inlineStr">
         <is>
           <t>Course presentation and video checkpoint</t>
         </is>
       </c>
-      <c r="C48" s="36" t="inlineStr">
+      <c r="C49" s="36" t="inlineStr">
         <is>
           <t>Deliver the course presentation/video using the reviewed evidence and acknowledged limitations.</t>
         </is>
       </c>
-      <c r="D48" s="13" t="inlineStr">
+      <c r="D49" s="13" t="inlineStr">
         <is>
           <t>34, 35</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="29" customHeight="1">
-      <c r="A49" s="8" t="inlineStr">
+    <row r="50" ht="29" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Research continuation</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="58" customHeight="1">
-      <c r="A50" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="B50" s="36" t="inlineStr">
-        <is>
-          <t>Further experiments and external validation</t>
-        </is>
-      </c>
-      <c r="C50" s="36" t="inlineStr">
-        <is>
-          <t>Select and run extensions justified by the reviewed evidence, biological relevance, collaborators and available resources. Includes the optional structure extension (plan item 6): sequence against sequence plus predicted structure features, only on tasks where structure plausibly acts.</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>29</t>
         </is>
       </c>
     </row>
     <row r="51" ht="58" customHeight="1">
       <c r="A51" s="13" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B51" s="36" t="inlineStr">
         <is>
-          <t>Consolidate manuscript and review publication readiness</t>
+          <t>Further experiments and external validation</t>
         </is>
       </c>
       <c r="C51" s="36" t="inlineStr">
         <is>
-          <t>Refine the manuscript already underway, integrate additional evidence and seek group feedback. Venue, submission date and final research end remain undecided.</t>
+          <t>Select and run extensions justified by the reviewed evidence, biological relevance, collaborators and available resources. In March, after the project's designs. Includes the optional structure extension (plan item 6): sequence against sequence plus predicted structure features, only on tasks where structure plausibly acts.</t>
         </is>
       </c>
       <c r="D51" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>21, 25, 29</t>
         </is>
       </c>
     </row>
     <row r="52" ht="58" customHeight="1">
       <c r="A52" s="13" t="n">
+        <v>39</v>
+      </c>
+      <c r="B52" s="36" t="inlineStr">
+        <is>
+          <t>Consolidate manuscript and review publication readiness</t>
+        </is>
+      </c>
+      <c r="C52" s="36" t="inlineStr">
+        <is>
+          <t>Refine the manuscript already underway, integrate additional evidence and seek group feedback. Venue, submission date and final research end remain undecided.</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="58" customHeight="1">
+      <c r="A53" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="B52" s="36" t="inlineStr">
+      <c r="B53" s="36" t="inlineStr">
         <is>
           <t>March research review and next-step decision</t>
         </is>
       </c>
-      <c r="C52" s="36" t="inlineStr">
+      <c r="C53" s="36" t="inlineStr">
         <is>
           <t>Review the evidence and decide whether to extend the experiments, revise the manuscript, prepare a submission or change direction. Adjust the timeline to the chosen next steps.</t>
         </is>
       </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="D53" s="13" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="24" customHeight="1">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-    </row>
-    <row r="54" ht="29" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+    </row>
+    <row r="55" ht="29" customHeight="1">
+      <c r="A55" s="8" t="inlineStr">
         <is>
           <t>Planning notes</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="34" customHeight="1">
-      <c r="A55" s="33" t="inlineStr">
+    <row r="56" ht="34" customHeight="1">
+      <c r="A56" s="33" t="inlineStr">
         <is>
           <t>Update the dates and corresponding week cells together in Gantt. Keep each task ID unchanged when editing its expected output or prerequisites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="42" customHeight="1">
-      <c r="A56" s="33" t="inlineStr">
-        <is>
-          <t>The team completed the initial six-paper review by September 21. Continued interpretation and discussion run through the October 7 meeting. September 21 start dates for current work are approximate planning anchors.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="33" t="inlineStr">
         <is>
-          <t>October 7 is the review with Mina and the target for a working alignment definition. Stage 1 includes the immediate revisions after that meeting. Future experiment dates are proposed windows.</t>
+          <t>The team completed the initial six-paper review by September 21. Continued interpretation and discussion run through the October 7 meeting. September 21 start dates for current work are approximate planning anchors.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="33" t="inlineStr">
         <is>
-          <t>Coupled Mamba is the priority architecture comparison. Optional layer/PCA, alignment-loss, additional DNA, RNA and protein encoder comparisons and the IsoFormer fusion comparison depend on earlier findings and available capacity. The tokenizer and collaborating group must first be identified with Julian.</t>
+          <t>October 7 is the review with Mina and the target for a working alignment definition. Stage 1 includes the immediate revisions after that meeting. Future experiment dates are proposed windows.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="42" customHeight="1">
       <c r="A59" s="33" t="inlineStr">
         <is>
-          <t>The bibliography, Research Canvas and project plan are due September 27 at 23:59 Eastern. December 1, 7 and 8 checkpoints come from the course schedule; confirm the corresponding WebCourses deadlines.</t>
+          <t>The research plan's items come first: its baselines (17, 24, 41, with IsoFormer as 44), the mRFP control (18) and its datasets (42). Coupled Mamba (20, 21) and IsoFormer-style cross-attention (25) follow from January and are scored against all of them. Optional layer/PCA and alignment-loss comparisons depend on earlier findings and available capacity. The tokenizer and collaborating group must first be identified with Julian.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="42" customHeight="1">
       <c r="A60" s="33" t="inlineStr">
         <is>
-          <t>AI supports implementation, paper discussion, analysis and writing throughout the project. Each research task includes interpreting its evidence and revising the resulting claims. OpenAI Codex organized the original plan; Claude assisted with the September 29 revision adding the DNA modality and the October 3 status update.</t>
+          <t>The bibliography, Research Canvas and project plan are due September 27 at 23:59 Eastern. December 1, 7 and 8 checkpoints come from the course schedule; confirm the corresponding WebCourses deadlines.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="42" customHeight="1">
       <c r="A61" s="33" t="inlineStr">
         <is>
+          <t>AI supports implementation, paper discussion, analysis and writing throughout the project. Each research task includes interpreting its evidence and revising the resulting claims. OpenAI Codex organized the original plan; Claude assisted with the September 29 revision adding the DNA modality, the October 3 status update and the October revisions that fold in Mina's research plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="42" customHeight="1">
+      <c r="A62" s="33" t="inlineStr">
+        <is>
           <t>Coordination began September 14. Stage 1 manuscript drafting begins September 26 and continues in Overleaf as the work develops. March is a planning horizon rather than a fixed research endpoint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="48" customHeight="1">
-      <c r="A62" s="33" t="inlineStr">
-        <is>
-          <t>Planning example: Mélot-Chesnel, Designing Trustworthy Generative AI Agents for Collaborative Decision Making (2026), section 4 and Figure 1, explicitly schedules reconsidering questions and hypotheses between studies. This informed retaining time for interpretation and revision. https://doi.org/10.3233/FAIA260562</t>
         </is>
       </c>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="33" t="inlineStr">
         <is>
+          <t>Planning example: Mélot-Chesnel, Designing Trustworthy Generative AI Agents for Collaborative Decision Making (2026), section 4 and Figure 1, explicitly schedules reconsidering questions and hypotheses between studies. This informed retaining time for interpretation and revision. https://doi.org/10.3233/FAIA260562</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="48" customHeight="1">
+      <c r="A64" s="33" t="inlineStr">
+        <is>
           <t>Planning example: UQ AGRC7617, Sequential mid-project assessment, uses a proposal and Gantt with supervisor discussion, followed by AI feedback on mature drafts. This illustrates review within planning. https://course-profiles.uq.edu.au/course-profiles/AGRC7617-62151-7660</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="33" t="inlineStr">
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="33" t="inlineStr">
         <is>
           <t>These examples informed the September 27 planning discussion. They do not establish CAP6942 requirements or measured AI time savings.</t>
         </is>
       </c>
-    </row>
-    <row r="65" ht="24" customHeight="1">
-      <c r="A65" s="2" t="n"/>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="n"/>
-      <c r="D65" s="2" t="n"/>
     </row>
     <row r="66" ht="24" customHeight="1">
       <c r="A66" s="2" t="n"/>
@@ -4379,26 +4443,32 @@
       <c r="C69" s="2" t="n"/>
       <c r="D69" s="2" t="n"/>
     </row>
+    <row r="70" ht="24" customHeight="1">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+      <c r="D70" s="2" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A62:D62"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A63:D63"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A44:D44"/>
     <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A54:D54"/>
-    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A50:D50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" tooltip="Open planning example" r:id="rId1"/>

</xml_diff>

<commit_message>
Stage 3 steps 3 and 4 results; sync notes, Gantt, deck and README to October 19
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01A54DUp2K2ADqzEJ7zvsPHg
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -600,7 +600,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 15, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan comes first (17, 18, 24, 41, 44, 42); Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
+          <t>As of October 19, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan comes first (17, 18, 24, 41, 44, 42); Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
         </is>
       </c>
     </row>
@@ -1605,9 +1605,9 @@
           <t>Harden single-model and simple-fusion baselines</t>
         </is>
       </c>
-      <c r="C24" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
@@ -1624,7 +1624,7 @@
       <c r="G24" s="13" t="str"/>
       <c r="H24" s="13" t="str"/>
       <c r="I24" s="13" t="str"/>
-      <c r="J24" s="37" t="inlineStr">
+      <c r="J24" s="23" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -1655,9 +1655,9 @@
           <t>Run matched BioLangFusion-style comparisons; reproduce BioLangFusion exactly on its five published datasets (plan item 1, Phase A)</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
@@ -1675,12 +1675,12 @@
       <c r="H25" s="13" t="n"/>
       <c r="I25" s="13" t="n"/>
       <c r="J25" s="13" t="n"/>
-      <c r="K25" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L25" s="37" t="inlineStr">
+      <c r="K25" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L25" s="23" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2229,9 +2229,9 @@
           <t>Repeat runs, quantify uncertainty and revise claims</t>
         </is>
       </c>
-      <c r="C36" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
@@ -2249,32 +2249,32 @@
       <c r="H36" s="13" t="str"/>
       <c r="I36" s="13" t="str"/>
       <c r="J36" s="13" t="str"/>
-      <c r="K36" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L36" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="M36" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="N36" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="O36" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P36" s="37" t="inlineStr">
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L36" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M36" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N36" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O36" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P36" s="23" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2353,9 +2353,9 @@
           <t>LucaOne frozen baseline on stability and GTEx, matched comparison (plan item 2)</t>
         </is>
       </c>
-      <c r="C38" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
@@ -2377,12 +2377,12 @@
       <c r="L38" s="13" t="n"/>
       <c r="M38" s="13" t="n"/>
       <c r="N38" s="13" t="n"/>
-      <c r="O38" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P38" s="37" t="inlineStr">
+      <c r="O38" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P38" s="23" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -2519,9 +2519,9 @@
           <t>IsoFormer's cross-attention aggregator reproduced on GTEx as a baseline, beside LucaOne (not on the plan's list)</t>
         </is>
       </c>
-      <c r="C41" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -2543,12 +2543,12 @@
       <c r="L41" s="13" t="n"/>
       <c r="M41" s="13" t="n"/>
       <c r="N41" s="13" t="n"/>
-      <c r="O41" s="37" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="P41" s="37" t="inlineStr">
+      <c r="O41" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P41" s="23" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -3358,12 +3358,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A45:Z45"/>
     <mergeCell ref="A23:Z23"/>
-    <mergeCell ref="A45:Z45"/>
+    <mergeCell ref="A42:Z42"/>
     <mergeCell ref="X5:Z5"/>
+    <mergeCell ref="A56:Z56"/>
     <mergeCell ref="A3:Z3"/>
-    <mergeCell ref="A56:Z56"/>
-    <mergeCell ref="A51:Z51"/>
     <mergeCell ref="A4:Z4"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A2:Z2"/>
@@ -3372,7 +3372,7 @@
     <mergeCell ref="A7:Z7"/>
     <mergeCell ref="J5:M5"/>
     <mergeCell ref="N5:R5"/>
-    <mergeCell ref="A42:Z42"/>
+    <mergeCell ref="A51:Z51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4451,24 +4451,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A50:D50"/>
     <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A63:D63"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A64:D64"/>
+    <mergeCell ref="A59:D59"/>
     <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A63:D63"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="A44:D44"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A64:D64"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A50:D50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" tooltip="Open planning example" r:id="rId1"/>

</xml_diff>

<commit_message>
Stage 4 round 1: mRFP control and BioLangFusion Phase A run, Phase B built; sync records, READMEs, Gantt and notes to October 20
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01A54DUp2K2ADqzEJ7zvsPHg
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,6 +258,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -600,7 +603,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 19, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan comes first (17, 18, 24, 41, 44, 42); Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
+          <t>As of October 20, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan comes first (17, 18, 24, 41, 44, 42); Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
         </is>
       </c>
     </row>
@@ -1709,9 +1712,9 @@
           <t>Repeat diagnostics and null/control comparisons, including the mRFP synonymous control (plan item 5)</t>
         </is>
       </c>
-      <c r="C26" s="24" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
@@ -1729,7 +1732,7 @@
       <c r="H26" s="13" t="str"/>
       <c r="I26" s="13" t="str"/>
       <c r="J26" s="13" t="str"/>
-      <c r="K26" s="37" t="inlineStr">
+      <c r="K26" s="42" t="inlineStr">
         <is>
           <t>██</t>
         </is>

</xml_diff>

<commit_message>
Sync the plan, notes, READMEs and deck to the October 22 results
Phase B's four swaps, LucaOne on stability, and the human half-life and
translation-efficiency probes all have results now, so every document that
described them as unrun has been updated.

The finding that changes the account: putting mRNA-FM in the RNA slot
raises E. coli by eight points as a single encoder, resolved, and the +6.9
fusion gain Phase A measured there falls to +0.3 [-2.9, +3.7]. The clearest
fusion win in the project was fusion compensating for a weak encoder.

Gantt: 41 and 42 move to in progress starting October 22; the Details sheet
records what each produced. Notes: the Stage 4 status paragraph, and
questions 2 and 5 rewritten around the new results. Deck: three new slides
for Phase B, LucaOne and the full-transcript tasks, 13 in all.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A54DUp2K2ADqzEJ7zvsPHg
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -603,7 +603,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 20, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan's priorities come first and are mapped to IDs here: item 1 Phase A to 17, item 1 Phase B to 24, item 2 to 41, items 3 and 4 to 42, item 5 to 18, item 6 to 38, item 7 to 43, with IsoFormer on GTEx as 44. Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
+          <t>As of October 22, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan's priorities come first and are mapped to IDs here: item 1 Phase A to 17, item 1 Phase B to 24, item 2 to 41, items 3 and 4 to 42, item 5 to 18, item 6 to 38, item 7 to 43, with IsoFormer on GTEx as 44. Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
         </is>
       </c>
     </row>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>Nov 9</t>
+          <t>Oct 22</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
@@ -2381,8 +2381,16 @@
       <c r="I38" s="13" t="n"/>
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n"/>
+      <c r="L38" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M38" s="23" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="23" t="inlineStr">
         <is>
@@ -2421,7 +2429,7 @@
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>Nov 23</t>
+          <t>Oct 22</t>
         </is>
       </c>
       <c r="E39" s="15" t="inlineStr">
@@ -2435,8 +2443,16 @@
       <c r="I39" s="13" t="n"/>
       <c r="J39" s="13" t="n"/>
       <c r="K39" s="13" t="n"/>
-      <c r="L39" s="13" t="n"/>
-      <c r="M39" s="13" t="n"/>
+      <c r="L39" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M39" s="37" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="N39" s="13" t="n"/>
       <c r="O39" s="13" t="n"/>
       <c r="P39" s="13" t="n"/>
@@ -3933,7 +3949,7 @@
       </c>
       <c r="C31" s="36" t="inlineStr">
         <is>
-          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM or other suitable codon models, mRNA-FM, ProtBERT, other DNA encoders; ESM-2 150M as a further protein candidate), then promising triples, on Fungal, E. coli, mRNA stability and Ab1 (CoV-Vac if feasible). Runs directly after the reproduction (17) and before LucaOne (41), in the plan's implementation order. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2. Built October 20 in Code/stage4/tier2_encoder_swaps.ipynb and extended to mRNA stability, which the plan names: eight swaps on CoV-Vac, fungal and E. coli, three on stability (mRNA-FM, CaLM, ESM-2 150M), about 53 GB of token cache in all. Chase runs it; Code/stage4/RUNBOOK.md has the order.</t>
+          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM or other suitable codon models, mRNA-FM, ProtBERT, other DNA encoders; ESM-2 150M as a further protein candidate), then promising triples, on Fungal, E. coli, mRNA stability and Ab1 (CoV-Vac if feasible). Runs directly after the reproduction (17) and before LucaOne (41), in the plan's implementation order. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2. Built October 20 in Code/stage4/tier2_encoder_swaps.ipynb and extended to mRNA stability, which the plan names: eight swaps on CoV-Vac, fungal and E. coli, three on stability (mRNA-FM, CaLM, ESM-2 150M), about 53 GB of token cache in all. Chase runs it; Code/stage4/RUNBOOK.md has the order. Four of the eight swaps ran on October 21 and 22 (CoV-Vac and E. coli, mRNA-FM and CaLM, seed 0). On E. coli the swapped encoder alone gains eight points, resolved, and the fusion gain Phase A measured there falls to +0.3 [-2.9, +3.7]. The DNA and protein swaps, RiNALMo, fungal, stability and seeds remain.</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -4053,7 +4069,7 @@
       </c>
       <c r="C37" s="36" t="inlineStr">
         <is>
-          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation. After the encoder swaps (24), in the plan's implementation order. Built October 20 in Code/stage4/tier2_lucaone_isoformer.ipynb. Stage 3 step 4 settled the scope: LucaOne's 1,280-token character-level context admits none of the GTEx DNA windows, so the baseline runs on mRNA stability only, as a ridge probe on frozen pooled vectors against BioLangFusion's own three encoders on the same split.</t>
+          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation. After the encoder swaps (24), in the plan's implementation order. Built October 20 in Code/stage4/tier2_lucaone_isoformer.ipynb. Stage 3 step 4 settled the scope: LucaOne's 1,280-token character-level context admits none of the GTEx DNA windows, so the baseline runs on mRNA stability only, as a ridge probe on frozen pooled vectors against BioLangFusion's own three encoders on the same split. Ran October 22 on mRNA stability: LucaOne's two streams score 0.483 against 0.390 for BioLangFusion's three encoders concatenated, +0.092 [+0.066, +0.120], resolved, under one matched ridge probe. GTEx stays ruled out by the context limit.</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
@@ -4073,7 +4089,7 @@
       </c>
       <c r="C38" s="36" t="inlineStr">
         <is>
-          <t>Plan items 3 and 4, each target run separately. Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Half-life: CDS only, CDS + 3' UTR, full transcript, and + protein. Translation efficiency: 5' UTR, CDS, full transcript, + protein, and the three-encoder fusion, with RiboNN as the external benchmark. Gain over the best full-transcript baseline. After the plan's baselines (24, 41, 44) and before the project's designs (20, 21), so every baseline is scored on these tasks. The feasibility gate is built in Code/stage4/tier3_halflife_te.ipynb and runs the week of October 20, ahead of this window: six mRNABench datasets, each checked for untranslated regions, a recoverable reading frame, labels and gene groups, with the composition floor measured per region set beside it.</t>
+          <t>Plan items 3 and 4, each target run separately. Gates first: 5' and 3' UTRs and coding-sequence coordinates present, labels and species present, grouped non-leaking splits; half-life, translation efficiency and ribosome load kept as separate targets. Half-life: CDS only, CDS + 3' UTR, full transcript, and + protein. Translation efficiency: 5' UTR, CDS, full transcript, + protein, and the three-encoder fusion, with RiboNN as the external benchmark. Gain over the best full-transcript baseline. After the plan's baselines (24, 41, 44) and before the project's designs (20, 21), so every baseline is scored on these tasks. The feasibility gate is built in Code/stage4/tier3_halflife_te.ipynb and runs the week of October 20, ahead of this window: six mRNABench datasets, each checked for untranslated regions, a recoverable reading frame, labels and gene groups, with the composition floor measured per region set beside it. The gate passed on all four primary datasets and the human half-life and translation-efficiency probes ran on October 22: full transcript with protein gains +0.053 and +0.030 over the best single encoder, which is the protein in both cases. The mouse sets are embedded and not yet scored, and the gains carry a standard error rather than a paired interval.</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Docs: Phase B complete (all eight swaps) in deck, guide, notes, run records; new figures
</commit_message>
<xml_diff>
--- a/docs/Research_Project_Plan_Gantt.xlsx
+++ b/docs/Research_Project_Plan_Gantt.xlsx
@@ -535,7 +535,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Z59"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="49" customWidth="1" min="2" max="2"/>
@@ -603,7 +603,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>As of October 22, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan's priorities come first and are mapped to IDs here: item 1 Phase A to 17, item 1 Phase B to 24, item 2 to 41, items 3 and 4 to 42, item 5 to 18, item 6 to 38, item 7 to 43, with IsoFormer on GTEx as 44. Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
+          <t>As of October 25, 2026. Fall weeks start Monday; January to March 2027 is a monthly horizon. The research plan's priorities come first and are mapped to IDs here: item 1 Phase A to 17, item 1 Phase B to 24, item 2 to 41, items 3 and 4 to 42, item 5 to 18, item 6 to 38, item 7 to 43, with IsoFormer on GTEx as 44. Coupled Mamba and cross-attention (20, 21, 25) follow from January.</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D70"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="49" customWidth="1" min="2" max="2"/>
@@ -3949,7 +3949,7 @@
       </c>
       <c r="C31" s="36" t="inlineStr">
         <is>
-          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM or other suitable codon models, mRNA-FM, ProtBERT, other DNA encoders; ESM-2 150M as a further protein candidate), then promising triples, on Fungal, E. coli, mRNA stability and Ab1 (CoV-Vac if feasible). Runs directly after the reproduction (17) and before LucaOne (41), in the plan's implementation order. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2. Built October 20 in Code/stage4/tier2_encoder_swaps.ipynb and extended to mRNA stability, which the plan names: eight swaps on CoV-Vac, fungal and E. coli, three on stability (mRNA-FM, CaLM, ESM-2 150M), about 53 GB of token cache in all. Chase runs it; Code/stage4/RUNBOOK.md has the order. Four of the eight swaps ran on October 21 and 22 (CoV-Vac and E. coli, mRNA-FM and CaLM, seed 0). On E. coli the swapped encoder alone gains eight points, resolved, and the fusion gain Phase A measured there falls to +0.3 [-2.9, +3.7]. The DNA and protein swaps, RiNALMo, fungal, stability and seeds remain.</t>
+          <t>Keep the reproduced BioLangFusion splits, grid, heads, TextCNN and evaluation fixed; replace one encoder at a time (CaLM or other suitable codon models, mRNA-FM, ProtBERT, other DNA encoders; ESM-2 150M as a further protein candidate), then promising triples, on Fungal, E. coli, mRNA stability and Ab1 (CoV-Vac if feasible). Runs directly after the reproduction (17) and before LucaOne (41), in the plan's implementation order. Report published, reproduced, best single, each head, each swap and Δfusion with seeds and paired differences. Now planned rather than conditional; the cleanest test of H2. Built October 20 in Code/stage4/tier2_encoder_swaps.ipynb and extended to mRNA stability, which the plan names: eight swaps on CoV-Vac, fungal and E. coli, three on stability (mRNA-FM, CaLM, ESM-2 150M), about 53 GB of token cache in all. Chase runs it; Code/stage4/RUNBOOK.md has the order. Four of the eight swaps ran on October 21 and 22 (CoV-Vac and E. coli, mRNA-FM and CaLM, seed 0). On E. coli the swapped encoder alone gains eight points, resolved, and the fusion gain Phase A measured there falls to +0.3 [-2.9, +3.7]. The DNA and protein swaps, RiNALMo, fungal, stability and seeds remain. Added at the October 22 review, as additions: fusion built around mRNA-FM (DNA with mRNA-FM, mRNA-FM with protein) and the other codon-level RNA encoders on the coding-sequence benchmarks, with cross-attention reported beside every swap; on the four swaps run, cross-attention is never better than the swapped encoder alone.</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="C37" s="36" t="inlineStr">
         <is>
-          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation. After the encoder swaps (24), in the plan's implementation order. Built October 20 in Code/stage4/tier2_lucaone_isoformer.ipynb. Stage 3 step 4 settled the scope: LucaOne's 1,280-token character-level context admits none of the GTEx DNA windows, so the baseline runs on mRNA stability only, as a ridge probe on frozen pooled vectors against BioLangFusion's own three encoders on the same split. Ran October 22 on mRNA stability: LucaOne's two streams score 0.483 against 0.390 for BioLangFusion's three encoders concatenated, +0.092 [+0.066, +0.120], resolved, under one matched ridge probe. GTEx stays ruled out by the context limit.</t>
+          <t>Verify LucaOne's input limits (1,280 tokens) and sequence types against the stability and GTEx files; extract frozen embeddings on the same folds and head as the fusion models; compare against the best single encoder and the best fused model; report cost and truncation. After the encoder swaps (24), in the plan's implementation order. Built October 20 in Code/stage4/tier2_lucaone_isoformer.ipynb. Stage 3 step 4 settled the scope: LucaOne's 1,280-token character-level context admits none of the GTEx DNA windows, so the baseline runs on mRNA stability only, as a ridge probe on frozen pooled vectors against BioLangFusion's own three encoders on the same split. Ran October 22 on mRNA stability: LucaOne's two streams score 0.483 against 0.390 for BioLangFusion's three encoders concatenated, +0.092 [+0.066, +0.120], resolved, under one matched ridge probe. GTEx stays ruled out by the context limit. Added at the October 22 review: the same matched-probe comparison on E. coli, CoV-Vac and fungal, which fit LucaOne's 1,280-token context after the 999-nucleotide rule.</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">

</xml_diff>